<commit_message>
Made edits to the model.xlsx file
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6fd52bb83a98f88c/Desktop/BUS 620 Economics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1605" documentId="8_{202E0E92-0A53-4DF2-844D-22EFC22CE560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55092676-ED51-4123-84A6-60FA2426361E}"/>
+  <xr:revisionPtr revIDLastSave="1854" documentId="8_{202E0E92-0A53-4DF2-844D-22EFC22CE560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62263D04-F852-4A7C-BB70-4D9BD7F68251}"/>
   <bookViews>
-    <workbookView xWindow="15" yWindow="60" windowWidth="22935" windowHeight="13935" xr2:uid="{CB3B63E6-161E-4EB6-9C62-E77ECB56D41C}"/>
+    <workbookView xWindow="15" yWindow="60" windowWidth="22935" windowHeight="13935" firstSheet="2" activeTab="6" xr2:uid="{CB3B63E6-161E-4EB6-9C62-E77ECB56D41C}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="8" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Checks" sheetId="4" r:id="rId4"/>
     <sheet name="Example Answer Report 1" sheetId="5" r:id="rId5"/>
     <sheet name="Example Answer Report 2" sheetId="7" r:id="rId6"/>
-    <sheet name="Hypothesis Answer Report " sheetId="6" r:id="rId7"/>
+    <sheet name="Hypothesis Report " sheetId="9" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="CARROT_BED_CAP">Inputs!$B$19</definedName>
@@ -153,7 +153,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="123">
   <si>
     <t>WEEKS</t>
   </si>
@@ -362,12 +362,6 @@
     <t>Total Labor Cost</t>
   </si>
   <si>
-    <t>Report Created: 10/9/2026 8:15:57 PM</t>
-  </si>
-  <si>
-    <t>Solution Time: 0.265 Seconds.</t>
-  </si>
-  <si>
     <t>Iterations: 0 Subproblems: 2</t>
   </si>
   <si>
@@ -522,6 +516,12 @@
   </si>
   <si>
     <t>Tolerance Result</t>
+  </si>
+  <si>
+    <t>Report Created: 10/14/2026 4:12:05 PM</t>
+  </si>
+  <si>
+    <t>Solution Time: 0.375 Seconds.</t>
   </si>
 </sst>
 </file>
@@ -623,7 +623,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -652,6 +652,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1000,16 +1007,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1020,108 +1027,108 @@
         <v>36</v>
       </c>
       <c r="C2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B3">
         <v>20000</v>
       </c>
       <c r="C3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B4">
         <v>64</v>
       </c>
       <c r="C4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B5">
         <v>720</v>
       </c>
       <c r="C5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B6">
         <v>34.72</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B7">
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B8">
         <v>1440</v>
       </c>
       <c r="C8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B9">
         <v>17.36</v>
       </c>
       <c r="C9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1132,72 +1139,72 @@
     </row>
     <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B12">
         <v>20</v>
       </c>
       <c r="C12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B13">
         <v>8800</v>
       </c>
       <c r="C13" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B14">
         <v>2.5</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B15">
         <v>880</v>
       </c>
       <c r="C15" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B16" s="2">
         <v>0.1</v>
       </c>
       <c r="C16" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -1208,72 +1215,72 @@
     </row>
     <row r="19" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B19">
         <v>20</v>
       </c>
       <c r="C19" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B20">
         <v>2094</v>
       </c>
       <c r="C20" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B21">
         <v>0.83299999999999996</v>
       </c>
       <c r="C21" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B22">
         <v>440</v>
       </c>
       <c r="C22" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B23" s="3">
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="C23" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -1284,72 +1291,72 @@
     </row>
     <row r="26" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B26">
         <v>30</v>
       </c>
       <c r="C26" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B27">
         <v>2700</v>
       </c>
       <c r="C27" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B28">
         <v>1.25</v>
       </c>
       <c r="C28" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B29">
         <v>880</v>
       </c>
       <c r="C29" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B30" s="3">
         <v>1.2500000000000001E-2</v>
       </c>
       <c r="C30" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1684,7 +1691,7 @@
     </row>
     <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B7">
         <f>Optimization!B1</f>
@@ -1693,7 +1700,7 @@
     </row>
     <row r="8" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B8" s="4" t="str">
         <f>IF(B6=B7,"PASS","FAIL")</f>
@@ -1713,7 +1720,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B11">
         <f>Optimization!B2</f>
@@ -1722,7 +1729,7 @@
     </row>
     <row r="12" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B12" s="4" t="str">
         <f>IF(B10=B11,"PASS","FAIL")</f>
@@ -1742,7 +1749,7 @@
     </row>
     <row r="15" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B15" s="4">
         <f>Optimization!B3</f>
@@ -1751,7 +1758,7 @@
     </row>
     <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B16" s="4" t="str">
         <f>IF(B14=B15,"PASS","FAIL")</f>
@@ -1763,7 +1770,7 @@
     </row>
     <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B18">
         <v>42762</v>
@@ -1771,7 +1778,7 @@
     </row>
     <row r="19" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B19" s="4">
         <f>Optimization!B7</f>
@@ -1780,7 +1787,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B20">
         <v>20</v>
@@ -1788,7 +1795,7 @@
     </row>
     <row r="21" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B21" t="str">
         <f>IF(ABS(B19-B18)&lt;=B20,"PASS","FAIL")</f>
@@ -2149,7 +2156,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2171,13 +2178,13 @@
     <row r="7" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:5" collapsed="1" x14ac:dyDescent="0.25">
@@ -2258,7 +2265,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B21" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
@@ -2396,7 +2403,7 @@
         <v>62</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G32" s="8">
         <v>0</v>
@@ -2416,7 +2423,7 @@
         <v>63</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G33" s="8">
         <v>0</v>
@@ -2436,7 +2443,7 @@
         <v>64</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G34" s="8">
         <v>0</v>
@@ -2458,9 +2465,9 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA2BB34E-83A8-4C9C-8F24-2AEF2CD56844}">
-  <dimension ref="A1:G35"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="1" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3335E638-4550-4578-AD93-BBAFED961797}">
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.28515625" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
@@ -2483,7 +2490,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>69</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2496,75 +2503,74 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" collapsed="1" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:5" collapsed="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="15" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="6">
-        <v>42775.155387742139</v>
-      </c>
-      <c r="E16" s="6">
+      <c r="D16" s="17">
+        <v>38227.058405064556</v>
+      </c>
+      <c r="E16" s="17">
         <v>42775.155387742139</v>
       </c>
     </row>
@@ -2574,217 +2580,207 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="15" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-    </row>
-    <row r="22" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="8" t="s">
+      <c r="B21" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C21" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D22" s="8">
+      <c r="D21" s="18">
+        <v>7</v>
+      </c>
+      <c r="E21" s="18">
         <v>10</v>
       </c>
-      <c r="E22" s="8">
+      <c r="F21" s="16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D22" s="18">
+        <v>20</v>
+      </c>
+      <c r="E22" s="18">
+        <v>20</v>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23" s="17">
+        <v>30</v>
+      </c>
+      <c r="E23" s="17">
+        <v>30</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E27" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="F27" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="G27" s="15" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D28" s="18">
+        <v>60</v>
+      </c>
+      <c r="E28" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="F28" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="G28" s="16">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="18">
+        <v>5276.8228463282185</v>
+      </c>
+      <c r="E29" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="F29" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="G29" s="16">
+        <v>1203.1771536717815</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B30" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="D30" s="18">
         <v>10</v>
       </c>
-      <c r="F22" s="8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="8" t="s">
+      <c r="E30" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="F30" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="G30" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C31" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D31" s="18">
         <v>20</v>
       </c>
-      <c r="E23" s="8">
-        <v>20</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="6" t="s">
+      <c r="E31" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="F31" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="G31" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B32" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C32" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D32" s="18">
         <v>30</v>
       </c>
-      <c r="E24" s="6">
-        <v>30</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" collapsed="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="E29" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B30" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D30" s="8">
-        <v>60</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="F30" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="G30" s="8">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B31" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D31" s="8">
-        <v>5276.8228463282185</v>
-      </c>
-      <c r="E31" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="F31" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="G31" s="8">
-        <v>1203.1771536717824</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B32" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="D32" s="8">
-        <v>10</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="G32" s="8">
+      <c r="E32" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="F32" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="G32" s="16">
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B33" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="D33" s="8">
-        <v>20</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="F33" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="G33" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B34" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="D34" s="8">
-        <v>30</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="F34" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="G34" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="6" t="s">
+    <row r="33" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="C35" s="6"/>
-      <c r="D35" s="6"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
-      <c r="G35" s="6"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update workbook with marginal cost schedules and validation checks
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6fd52bb83a98f88c/Desktop/BUS 620 Economics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1854" documentId="8_{202E0E92-0A53-4DF2-844D-22EFC22CE560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62263D04-F852-4A7C-BB70-4D9BD7F68251}"/>
+  <xr:revisionPtr revIDLastSave="1997" documentId="8_{202E0E92-0A53-4DF2-844D-22EFC22CE560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1297A18D-1302-4989-A597-7C0EDDDF2F14}"/>
   <bookViews>
-    <workbookView xWindow="15" yWindow="60" windowWidth="22935" windowHeight="13935" firstSheet="2" activeTab="6" xr2:uid="{CB3B63E6-161E-4EB6-9C62-E77ECB56D41C}"/>
+    <workbookView xWindow="105" yWindow="705" windowWidth="22935" windowHeight="13935" firstSheet="5" activeTab="8" xr2:uid="{CB3B63E6-161E-4EB6-9C62-E77ECB56D41C}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="8" r:id="rId1"/>
@@ -20,6 +20,8 @@
     <sheet name="Example Answer Report 1" sheetId="5" r:id="rId5"/>
     <sheet name="Example Answer Report 2" sheetId="7" r:id="rId6"/>
     <sheet name="Hypothesis Report " sheetId="9" r:id="rId7"/>
+    <sheet name="Marginal Cost" sheetId="10" r:id="rId8"/>
+    <sheet name="Cost Structure" sheetId="11" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="CARROT_BED_CAP">Inputs!$B$19</definedName>
@@ -153,7 +155,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="137">
   <si>
     <t>WEEKS</t>
   </si>
@@ -522,13 +524,55 @@
   </si>
   <si>
     <t>Solution Time: 0.375 Seconds.</t>
+  </si>
+  <si>
+    <t>Tomato Marginal Cost Schedule</t>
+  </si>
+  <si>
+    <t>Total Cost</t>
+  </si>
+  <si>
+    <t>Marginal Cost</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Carrot Marginal  Cost Schedule</t>
+  </si>
+  <si>
+    <t>Mesclun Marginal Cost Schedule</t>
+  </si>
+  <si>
+    <t>Expxected Max Beds</t>
+  </si>
+  <si>
+    <t>Actual Beds Used</t>
+  </si>
+  <si>
+    <t>Beds Result</t>
+  </si>
+  <si>
+    <t>Expected Max Labor</t>
+  </si>
+  <si>
+    <t>Actual Labor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Labor Result </t>
+  </si>
+  <si>
+    <t>Total Fertilizer Cost</t>
+  </si>
+  <si>
+    <t>Fixed Cost</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -565,8 +609,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -576,6 +627,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -623,7 +680,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -652,13 +709,15 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1641,10 +1700,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0213E619-8C1A-4944-B8AD-22830FD50E6A}">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.140625" customWidth="1"/>
+    <col min="1" max="1" width="21" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -1799,6 +1858,58 @@
       </c>
       <c r="B21" t="str">
         <f>IF(ABS(B19-B18)&lt;=B20,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="B23">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="B24">
+        <f>Optimization!B5</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="B25" t="str">
+        <f>IF(B24&lt;=B23,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="B27">
+        <v>6480</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B28">
+        <f>Optimization!B6</f>
+        <v>5276.8228463282185</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="B29" t="str">
+        <f>IF(B28&lt;=B27,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>
@@ -2547,30 +2658,30 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="7" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="17">
+      <c r="D16" s="6">
         <v>38227.058405064556</v>
       </c>
-      <c r="E16" s="17">
+      <c r="E16" s="6">
         <v>42775.155387742139</v>
       </c>
     </row>
@@ -2580,70 +2691,70 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E20" s="15" t="s">
+      <c r="E20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="F20" s="15" t="s">
+      <c r="F20" s="7" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C21" s="16" t="s">
+      <c r="C21" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="18">
+      <c r="D21" s="8">
         <v>7</v>
       </c>
-      <c r="E21" s="18">
+      <c r="E21" s="8">
         <v>10</v>
       </c>
-      <c r="F21" s="16" t="s">
+      <c r="F21" s="8" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C22" s="16" t="s">
+      <c r="C22" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="D22" s="18">
+      <c r="D22" s="8">
         <v>20</v>
       </c>
-      <c r="E22" s="18">
+      <c r="E22" s="8">
         <v>20</v>
       </c>
-      <c r="F22" s="16" t="s">
+      <c r="F22" s="8" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="14" t="s">
+      <c r="B23" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="14" t="s">
+      <c r="C23" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D23" s="17">
+      <c r="D23" s="6">
         <v>30</v>
       </c>
-      <c r="E23" s="17">
+      <c r="E23" s="6">
         <v>30</v>
       </c>
-      <c r="F23" s="14" t="s">
+      <c r="F23" s="6" t="s">
         <v>47</v>
       </c>
     </row>
@@ -2653,134 +2764,1202 @@
       </c>
     </row>
     <row r="27" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="15" t="s">
+      <c r="B27" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C27" s="15" t="s">
+      <c r="C27" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="D27" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E27" s="15" t="s">
+      <c r="E27" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F27" s="15" t="s">
+      <c r="F27" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G27" s="15" t="s">
+      <c r="G27" s="7" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B28" s="16" t="s">
+      <c r="B28" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D28" s="18">
+      <c r="D28" s="8">
         <v>60</v>
       </c>
-      <c r="E28" s="16" t="s">
+      <c r="E28" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="F28" s="16" t="s">
+      <c r="F28" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="G28" s="16">
+      <c r="G28" s="8">
         <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B29" s="16" t="s">
+      <c r="B29" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C29" s="16" t="s">
+      <c r="C29" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D29" s="18">
+      <c r="D29" s="8">
         <v>5276.8228463282185</v>
       </c>
-      <c r="E29" s="16" t="s">
+      <c r="E29" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="F29" s="16" t="s">
+      <c r="F29" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="G29" s="16">
+      <c r="G29" s="8">
         <v>1203.1771536717815</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B30" s="16" t="s">
+      <c r="B30" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C30" s="16" t="s">
+      <c r="C30" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D30" s="18">
+      <c r="D30" s="8">
         <v>10</v>
       </c>
-      <c r="E30" s="16" t="s">
+      <c r="E30" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F30" s="16" t="s">
+      <c r="F30" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="G30" s="16">
+      <c r="G30" s="8">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B31" s="16" t="s">
+      <c r="B31" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C31" s="16" t="s">
+      <c r="C31" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="D31" s="18">
+      <c r="D31" s="8">
         <v>20</v>
       </c>
-      <c r="E31" s="16" t="s">
+      <c r="E31" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="F31" s="16" t="s">
+      <c r="F31" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="G31" s="16">
+      <c r="G31" s="8">
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B32" s="16" t="s">
+      <c r="B32" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C32" s="16" t="s">
+      <c r="C32" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D32" s="18">
+      <c r="D32" s="8">
         <v>30</v>
       </c>
-      <c r="E32" s="16" t="s">
+      <c r="E32" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F32" s="16" t="s">
+      <c r="F32" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="G32" s="16">
+      <c r="G32" s="8">
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="14" t="s">
+      <c r="B33" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6D619FE-79F3-4F8F-A3C4-E7E7F8031B48}">
+  <dimension ref="A1:C78"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.28515625" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <f>(A3*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A3)*FARMER_RATE</f>
+        <v>3437.28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <f>(A4*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A4)*FARMER_RATE</f>
+        <v>7562.0160000000014</v>
+      </c>
+      <c r="C4" s="4">
+        <f>B4-B3</f>
+        <v>4124.7360000000008</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <f>(A5*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A5)*FARMER_RATE</f>
+        <v>12477.326400000004</v>
+      </c>
+      <c r="C5" s="4">
+        <f t="shared" ref="C5:C22" si="0">B5-B4</f>
+        <v>4915.3104000000021</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <f>(A6*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A6)*FARMER_RATE</f>
+        <v>18300.078720000005</v>
+      </c>
+      <c r="C6" s="4">
+        <f t="shared" si="0"/>
+        <v>5822.7523200000014</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <f>(A7*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A7)*FARMER_RATE</f>
+        <v>25162.608240000009</v>
+      </c>
+      <c r="C7" s="4">
+        <f t="shared" si="0"/>
+        <v>6862.5295200000037</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <f>(A8*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A8)*FARMER_RATE</f>
+        <v>33214.642876800011</v>
+      </c>
+      <c r="C8" s="4">
+        <f t="shared" si="0"/>
+        <v>8052.0346368000028</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <f>(A9*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A9)*FARMER_RATE</f>
+        <v>42625.458358560019</v>
+      </c>
+      <c r="C9" s="4">
+        <f t="shared" si="0"/>
+        <v>9410.815481760008</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <f>(A10*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A10)*FARMER_RATE</f>
+        <v>53586.290507904028</v>
+      </c>
+      <c r="C10" s="4">
+        <f t="shared" si="0"/>
+        <v>10960.832149344009</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <f>(A11*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A11)*FARMER_RATE</f>
+        <v>66313.034503531235</v>
+      </c>
+      <c r="C11" s="4">
+        <f t="shared" si="0"/>
+        <v>12726.743995627206</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <f>(A12*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A12)*FARMER_RATE</f>
+        <v>81049.264393204867</v>
+      </c>
+      <c r="C12" s="4">
+        <f t="shared" si="0"/>
+        <v>14736.229889673632</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <f>(A13*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A13)*FARMER_RATE</f>
+        <v>98069.609915777881</v>
+      </c>
+      <c r="C13" s="4">
+        <f t="shared" si="0"/>
+        <v>17020.345522573014</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>12</v>
+      </c>
+      <c r="B14">
+        <f>(A14*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A14)*FARMER_RATE</f>
+        <v>117683.53189893346</v>
+      </c>
+      <c r="C14" s="4">
+        <f t="shared" si="0"/>
+        <v>19613.921983155582</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15">
+        <f>(A15*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A15)*FARMER_RATE</f>
+        <v>140239.54217956238</v>
+      </c>
+      <c r="C15" s="4">
+        <f t="shared" si="0"/>
+        <v>22556.010280628921</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>14</v>
+      </c>
+      <c r="B16">
+        <f>(A16*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A16)*FARMER_RATE</f>
+        <v>166129.91919732778</v>
+      </c>
+      <c r="C16" s="4">
+        <f t="shared" si="0"/>
+        <v>25890.377017765393</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>15</v>
+      </c>
+      <c r="B17">
+        <f>(A17*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A17)*FARMER_RATE</f>
+        <v>195795.97619685059</v>
+      </c>
+      <c r="C17" s="4">
+        <f t="shared" si="0"/>
+        <v>29666.056999522814</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <f>(A18*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A18)*FARMER_RATE</f>
+        <v>229733.94540430469</v>
+      </c>
+      <c r="C18" s="4">
+        <f t="shared" si="0"/>
+        <v>33937.969207454094</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>17</v>
+      </c>
+      <c r="B19">
+        <f>(A19*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A19)*FARMER_RATE</f>
+        <v>268501.54869128112</v>
+      </c>
+      <c r="C19" s="4">
+        <f t="shared" si="0"/>
+        <v>38767.603286976431</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>18</v>
+      </c>
+      <c r="B20">
+        <f>(A20*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A20)*FARMER_RATE</f>
+        <v>312725.33318160975</v>
+      </c>
+      <c r="C20" s="4">
+        <f t="shared" si="0"/>
+        <v>44223.784490328631</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>19</v>
+      </c>
+      <c r="B21">
+        <f>(A21*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A21)*FARMER_RATE</f>
+        <v>363108.85908309149</v>
+      </c>
+      <c r="C21" s="4">
+        <f t="shared" si="0"/>
+        <v>50383.525901481742</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>20</v>
+      </c>
+      <c r="B22">
+        <f>(A22*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A22)*FARMER_RATE</f>
+        <v>420441.83683305327</v>
+      </c>
+      <c r="C22" s="4">
+        <f t="shared" si="0"/>
+        <v>57332.977749961778</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="14" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>1</v>
+      </c>
+      <c r="B26">
+        <f>(A26*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A26)*FARMER_RATE</f>
+        <v>1067.2129439999999</v>
+      </c>
+      <c r="C26" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>2</v>
+      </c>
+      <c r="B27">
+        <f>(A27*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A27)*FARMER_RATE</f>
+        <v>2187.7865351999994</v>
+      </c>
+      <c r="C27" s="4">
+        <f>B27-B26</f>
+        <v>1120.5735911999996</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>3</v>
+      </c>
+      <c r="B28">
+        <f>(A28*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A28)*FARMER_RATE</f>
+        <v>3363.7217978699991</v>
+      </c>
+      <c r="C28" s="4">
+        <f t="shared" ref="C28:C45" si="1">B28-B27</f>
+        <v>1175.9352626699997</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>4</v>
+      </c>
+      <c r="B29">
+        <f>(A29*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A29)*FARMER_RATE</f>
+        <v>4597.0864570889989</v>
+      </c>
+      <c r="C29" s="4">
+        <f t="shared" si="1"/>
+        <v>1233.3646592189998</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>5</v>
+      </c>
+      <c r="B30">
+        <f>(A30*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A30)*FARMER_RATE</f>
+        <v>5890.0170231452794</v>
+      </c>
+      <c r="C30" s="4">
+        <f t="shared" si="1"/>
+        <v>1292.9305660562804</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>6</v>
+      </c>
+      <c r="B31">
+        <f>(A31*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A31)*FARMER_RATE</f>
+        <v>7244.7209384686921</v>
+      </c>
+      <c r="C31" s="4">
+        <f t="shared" si="1"/>
+        <v>1354.7039153234127</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>7</v>
+      </c>
+      <c r="B32">
+        <f>(A32*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A32)*FARMER_RATE</f>
+        <v>8663.4787889188119</v>
+      </c>
+      <c r="C32" s="4">
+        <f t="shared" si="1"/>
+        <v>1418.7578504501198</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>8</v>
+      </c>
+      <c r="B33">
+        <f>(A33*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A33)*FARMER_RATE</f>
+        <v>10148.646581304893</v>
+      </c>
+      <c r="C33" s="4">
+        <f t="shared" si="1"/>
+        <v>1485.1677923860807</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>9</v>
+      </c>
+      <c r="B34">
+        <f>(A34*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A34)*FARMER_RATE</f>
+        <v>11702.658089067203</v>
+      </c>
+      <c r="C34" s="4">
+        <f t="shared" si="1"/>
+        <v>1554.0115077623104</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>10</v>
+      </c>
+      <c r="B35">
+        <f>(A35*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A35)*FARMER_RATE</f>
+        <v>13328.027268104315</v>
+      </c>
+      <c r="C35" s="4">
+        <f t="shared" si="1"/>
+        <v>1625.3691790371122</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>11</v>
+      </c>
+      <c r="B36">
+        <f>(A36*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A36)*FARMER_RATE</f>
+        <v>15027.350744787615</v>
+      </c>
+      <c r="C36" s="4">
+        <f t="shared" si="1"/>
+        <v>1699.3234766832993</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>12</v>
+      </c>
+      <c r="B37">
+        <f>(A37*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A37)*FARMER_RATE</f>
+        <v>16803.310378262511</v>
+      </c>
+      <c r="C37" s="4">
+        <f t="shared" si="1"/>
+        <v>1775.9596334748967</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>13</v>
+      </c>
+      <c r="B38">
+        <f>(A38*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A38)*FARMER_RATE</f>
+        <v>18658.675899195663</v>
+      </c>
+      <c r="C38" s="4">
+        <f t="shared" si="1"/>
+        <v>1855.3655209331519</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>14</v>
+      </c>
+      <c r="B39">
+        <f>(A39*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A39)*FARMER_RATE</f>
+        <v>20596.30762718906</v>
+      </c>
+      <c r="C39" s="4">
+        <f t="shared" si="1"/>
+        <v>1937.6317279933974</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>15</v>
+      </c>
+      <c r="B40">
+        <f>(A40*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A40)*FARMER_RATE</f>
+        <v>22619.15926914513</v>
+      </c>
+      <c r="C40" s="4">
+        <f t="shared" si="1"/>
+        <v>2022.8516419560692</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>16</v>
+      </c>
+      <c r="B41">
+        <f>(A41*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A41)*FARMER_RATE</f>
+        <v>24730.280800932007</v>
+      </c>
+      <c r="C41" s="4">
+        <f t="shared" si="1"/>
+        <v>2111.1215317868773</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>17</v>
+      </c>
+      <c r="B42">
+        <f>(A42*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A42)*FARMER_RATE</f>
+        <v>26932.82143476501</v>
+      </c>
+      <c r="C42" s="4">
+        <f t="shared" si="1"/>
+        <v>2202.5406338330031</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>18</v>
+      </c>
+      <c r="B43">
+        <f>(A43*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A43)*FARMER_RATE</f>
+        <v>29230.032674789087</v>
+      </c>
+      <c r="C43" s="4">
+        <f t="shared" si="1"/>
+        <v>2297.2112400240767</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>19</v>
+      </c>
+      <c r="B44">
+        <f>(A44*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A44)*FARMER_RATE</f>
+        <v>31625.271463417637</v>
+      </c>
+      <c r="C44" s="4">
+        <f t="shared" si="1"/>
+        <v>2395.2387886285505</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>20</v>
+      </c>
+      <c r="B45">
+        <f>(A45*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A45)*FARMER_RATE</f>
+        <v>34122.003421055866</v>
+      </c>
+      <c r="C45" s="4">
+        <f t="shared" si="1"/>
+        <v>2496.7319576382288</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A47" s="15" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A48" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>1</v>
+      </c>
+      <c r="B49">
+        <f>((A49*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A49)*FARMER_RATE)
++(A49*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>2461.9299999999998</v>
+      </c>
+      <c r="C49" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>2</v>
+      </c>
+      <c r="B50">
+        <f>((A50*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A50)*FARMER_RATE)
++(A50*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>4963.4082499999995</v>
+      </c>
+      <c r="C50" s="4">
+        <f>B50-B49</f>
+        <v>2501.4782499999997</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>3</v>
+      </c>
+      <c r="B51">
+        <f>((A51*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A51)*FARMER_RATE)
++(A51*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>7505.1762796874991</v>
+      </c>
+      <c r="C51" s="4">
+        <f t="shared" ref="C51:C78" si="2">B51-B50</f>
+        <v>2541.7680296874996</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>4</v>
+      </c>
+      <c r="B52">
+        <f>((A52*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A52)*FARMER_RATE)
++(A52*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>10087.987977578125</v>
+      </c>
+      <c r="C52" s="4">
+        <f t="shared" si="2"/>
+        <v>2582.8116978906255</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>5</v>
+      </c>
+      <c r="B53">
+        <f>((A53*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A53)*FARMER_RATE)
++(A53*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>12712.609784122313</v>
+      </c>
+      <c r="C53" s="4">
+        <f t="shared" si="2"/>
+        <v>2624.6218065441881</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>6</v>
+      </c>
+      <c r="B54">
+        <f>((A54*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A54)*FARMER_RATE)
++(A54*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>15379.820887708611</v>
+      </c>
+      <c r="C54" s="4">
+        <f t="shared" si="2"/>
+        <v>2667.2111035862981</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>7</v>
+      </c>
+      <c r="B55">
+        <f>((A55*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A55)*FARMER_RATE)
++(A55*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>18090.413423605794</v>
+      </c>
+      <c r="C55" s="4">
+        <f t="shared" si="2"/>
+        <v>2710.5925358971836</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>8</v>
+      </c>
+      <c r="B56">
+        <f>((A56*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A56)*FARMER_RATE)
++(A56*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>20845.192675886705</v>
+      </c>
+      <c r="C56" s="4">
+        <f t="shared" si="2"/>
+        <v>2754.7792522809104</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>9</v>
+      </c>
+      <c r="B57">
+        <f>((A57*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A57)*FARMER_RATE)
++(A57*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>23644.9772823772</v>
+      </c>
+      <c r="C57" s="4">
+        <f t="shared" si="2"/>
+        <v>2799.7846064904952</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>10</v>
+      </c>
+      <c r="B58">
+        <f>((A58*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A58)*FARMER_RATE)
++(A58*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>26490.599442674353</v>
+      </c>
+      <c r="C58" s="4">
+        <f t="shared" si="2"/>
+        <v>2845.6221602971527</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>11</v>
+      </c>
+      <c r="B59">
+        <f>((A59*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A59)*FARMER_RATE)
++(A59*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>29382.905129278555</v>
+      </c>
+      <c r="C59" s="4">
+        <f t="shared" si="2"/>
+        <v>2892.3056866042025</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>12</v>
+      </c>
+      <c r="B60">
+        <f>((A60*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A60)*FARMER_RATE)
++(A60*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>32322.754301884954</v>
+      </c>
+      <c r="C60" s="4">
+        <f t="shared" si="2"/>
+        <v>2939.8491726063985</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>13</v>
+      </c>
+      <c r="B61">
+        <f>((A61*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A61)*FARMER_RATE)
++(A61*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>35311.021124880055</v>
+      </c>
+      <c r="C61" s="4">
+        <f t="shared" si="2"/>
+        <v>2988.2668229951014</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>14</v>
+      </c>
+      <c r="B62">
+        <f>((A62*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A62)*FARMER_RATE)
++(A62*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>38348.59418809037</v>
+      </c>
+      <c r="C62" s="4">
+        <f t="shared" si="2"/>
+        <v>3037.573063210315</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>15</v>
+      </c>
+      <c r="B63">
+        <f>((A63*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A63)*FARMER_RATE)
++(A63*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>41436.376730830176</v>
+      </c>
+      <c r="C63" s="4">
+        <f t="shared" si="2"/>
+        <v>3087.7825427398056</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>16</v>
+      </c>
+      <c r="B64">
+        <f>((A64*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A64)*FARMER_RATE)
++(A64*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>44575.2868692966</v>
+      </c>
+      <c r="C64" s="4">
+        <f t="shared" si="2"/>
+        <v>3138.9101384664245</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>17</v>
+      </c>
+      <c r="B65">
+        <f>((A65*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A65)*FARMER_RATE)
++(A65*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>47766.257827360474</v>
+      </c>
+      <c r="C65" s="4">
+        <f t="shared" si="2"/>
+        <v>3190.9709580638737</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>18</v>
+      </c>
+      <c r="B66">
+        <f>((A66*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A66)*FARMER_RATE)
++(A66*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>51010.23817080263</v>
+      </c>
+      <c r="C66" s="4">
+        <f t="shared" si="2"/>
+        <v>3243.9803434421556</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>19</v>
+      </c>
+      <c r="B67">
+        <f>((A67*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A67)*FARMER_RATE)
++(A67*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>54308.192045045304</v>
+      </c>
+      <c r="C67" s="4">
+        <f t="shared" si="2"/>
+        <v>3297.9538742426739</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>20</v>
+      </c>
+      <c r="B68">
+        <f>((A68*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A68)*FARMER_RATE)
++(A68*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>57661.099416429868</v>
+      </c>
+      <c r="C68" s="4">
+        <f t="shared" si="2"/>
+        <v>3352.9073713845646</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>21</v>
+      </c>
+      <c r="B69">
+        <f>((A69*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A69)*FARMER_RATE)
++(A69*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>61069.956317091994</v>
+      </c>
+      <c r="C69" s="4">
+        <f t="shared" si="2"/>
+        <v>3408.8569006621256</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>22</v>
+      </c>
+      <c r="B70">
+        <f>((A70*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A70)*FARMER_RATE)
++(A70*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>64535.775093486867</v>
+      </c>
+      <c r="C70" s="4">
+        <f t="shared" si="2"/>
+        <v>3465.8187763948736</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>23</v>
+      </c>
+      <c r="B71">
+        <f>((A71*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A71)*FARMER_RATE)
++(A71*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>68059.584658617066</v>
+      </c>
+      <c r="C71" s="4">
+        <f t="shared" si="2"/>
+        <v>3523.8095651301992</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>24</v>
+      </c>
+      <c r="B72">
+        <f>((A72*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A72)*FARMER_RATE)
++(A72*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>71642.430748017156</v>
+      </c>
+      <c r="C72" s="4">
+        <f t="shared" si="2"/>
+        <v>3582.8460894000891</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>25</v>
+      </c>
+      <c r="B73">
+        <f>((A73*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A73)*FARMER_RATE)
++(A73*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>75285.376179549348</v>
+      </c>
+      <c r="C73" s="4">
+        <f t="shared" si="2"/>
+        <v>3642.9454315321927</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>26</v>
+      </c>
+      <c r="B74">
+        <f>((A74*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A74)*FARMER_RATE)
++(A74*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>78989.501117065476</v>
+      </c>
+      <c r="C74" s="4">
+        <f t="shared" si="2"/>
+        <v>3704.1249375161278</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>27</v>
+      </c>
+      <c r="B75">
+        <f>((A75*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A75)*FARMER_RATE)
++(A75*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>82755.903337991418</v>
+      </c>
+      <c r="C75" s="4">
+        <f t="shared" si="2"/>
+        <v>3766.4022209259419</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>28</v>
+      </c>
+      <c r="B76">
+        <f>((A76*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A76)*FARMER_RATE)
++(A76*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>86585.698504890999</v>
+      </c>
+      <c r="C76" s="4">
+        <f t="shared" si="2"/>
+        <v>3829.7951668995811</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>29</v>
+      </c>
+      <c r="B77">
+        <f>((A77*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A77)*FARMER_RATE)
++(A77*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>90480.020441066488</v>
+      </c>
+      <c r="C77" s="4">
+        <f t="shared" si="2"/>
+        <v>3894.3219361754891</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>30</v>
+      </c>
+      <c r="B78">
+        <f>((A78*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A78)*FARMER_RATE)
++(A78*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>94440.021410255009</v>
+      </c>
+      <c r="C78" s="4">
+        <f t="shared" si="2"/>
+        <v>3960.0009691885207</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7B837CD-71B5-41FE-AB68-B192F153FF71}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.140625" customWidth="1"/>
+    <col min="2" max="2" width="25.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="1">
+        <f>MIN(Calculations!B8,FARMER_HOURS)*FARMER_RATE</f>
+        <v>24998.399999999998</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="1">
+        <f>MAX(0,Calculations!B8-FARMER_HOURS)*TEMP_WORKER_RATE</f>
+        <v>79106.444612257867</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="1">
+        <f>Calculations!B22</f>
+        <v>104104.84461225786</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="1">
+        <f>Calculations!B18</f>
+        <v>44000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5">
+        <f>FIXED_COSTS</f>
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B6">
+        <f>SUM(B3:B5)</f>
+        <v>168104.84461225785</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update marginal cost schedules and pricing rules
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6fd52bb83a98f88c/Desktop/BUS 620 Economics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1997" documentId="8_{202E0E92-0A53-4DF2-844D-22EFC22CE560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1297A18D-1302-4989-A597-7C0EDDDF2F14}"/>
+  <xr:revisionPtr revIDLastSave="2068" documentId="8_{202E0E92-0A53-4DF2-844D-22EFC22CE560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04736648-7896-4C13-B99A-77F5A00D15DE}"/>
   <bookViews>
-    <workbookView xWindow="105" yWindow="705" windowWidth="22935" windowHeight="13935" firstSheet="5" activeTab="8" xr2:uid="{CB3B63E6-161E-4EB6-9C62-E77ECB56D41C}"/>
+    <workbookView xWindow="0" yWindow="450" windowWidth="22935" windowHeight="13935" firstSheet="5" activeTab="7" xr2:uid="{CB3B63E6-161E-4EB6-9C62-E77ECB56D41C}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="8" r:id="rId1"/>
@@ -155,7 +155,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="139">
   <si>
     <t>WEEKS</t>
   </si>
@@ -566,6 +566,12 @@
   </si>
   <si>
     <t>Fixed Cost</t>
+  </si>
+  <si>
+    <t>Beds (q)</t>
+  </si>
+  <si>
+    <t>Labor Hours</t>
   </si>
 </sst>
 </file>
@@ -680,7 +686,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -717,6 +723,13 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2900,997 +2913,1350 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6D619FE-79F3-4F8F-A3C4-E7E7F8031B48}">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:E84"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.28515625" customWidth="1"/>
     <col min="2" max="2" width="11.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B2" s="11" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+    </row>
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C3" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="D3" s="11" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="E3" s="11"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>0</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>1</v>
       </c>
-      <c r="B3">
-        <f>(A3*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A3)*FARMER_RATE</f>
-        <v>3437.28</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B5">
+        <f>(MIN(C5,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C5-FARMER_HOURS)*TEMP_WORKER_RATE)+(A5*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C5-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A5*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>5197.2800000000007</v>
+      </c>
+      <c r="C5">
+        <f>A5*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A5</f>
+        <v>99.000000000000014</v>
+      </c>
+      <c r="D5" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4">
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>2</v>
       </c>
-      <c r="B4">
-        <f>(A4*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A4)*FARMER_RATE</f>
-        <v>7562.0160000000014</v>
-      </c>
-      <c r="C4" s="4">
-        <f>B4-B3</f>
-        <v>4124.7360000000008</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="B6">
+        <f>(MIN(C6,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C6-FARMER_HOURS)*TEMP_WORKER_RATE)+(A6*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C6-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A6*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>11082.016000000001</v>
+      </c>
+      <c r="C6">
+        <f>A6*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A6</f>
+        <v>217.80000000000004</v>
+      </c>
+      <c r="D6" s="4">
+        <f>B6-B5</f>
+        <v>5884.7360000000008</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>3</v>
       </c>
-      <c r="B5">
-        <f>(A5*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A5)*FARMER_RATE</f>
-        <v>12477.326400000004</v>
-      </c>
-      <c r="C5" s="4">
-        <f t="shared" ref="C5:C22" si="0">B5-B4</f>
-        <v>4915.3104000000021</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="B7">
+        <f>(MIN(C7,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C7-FARMER_HOURS)*TEMP_WORKER_RATE)+(A7*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C7-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A7*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>17757.326400000005</v>
+      </c>
+      <c r="C7">
+        <f>A7*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A7</f>
+        <v>359.37000000000012</v>
+      </c>
+      <c r="D7" s="4">
+        <f t="shared" ref="D7:D24" si="0">B7-B6</f>
+        <v>6675.3104000000039</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>4</v>
       </c>
-      <c r="B6">
-        <f>(A6*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A6)*FARMER_RATE</f>
-        <v>18300.078720000005</v>
-      </c>
-      <c r="C6" s="4">
+      <c r="B8">
+        <f>(MIN(C8,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C8-FARMER_HOURS)*TEMP_WORKER_RATE)+(A8*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C8-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A8*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>25340.078720000005</v>
+      </c>
+      <c r="C8">
+        <f>A8*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A8</f>
+        <v>527.07600000000014</v>
+      </c>
+      <c r="D8" s="4">
         <f t="shared" si="0"/>
-        <v>5822.7523200000014</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7">
+        <v>7582.7523199999996</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>5</v>
       </c>
-      <c r="B7">
-        <f>(A7*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A7)*FARMER_RATE</f>
-        <v>25162.608240000009</v>
-      </c>
-      <c r="C7" s="4">
+      <c r="B9">
+        <f>(MIN(C9,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C9-FARMER_HOURS)*TEMP_WORKER_RATE)+(A9*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C9-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A9*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>33962.608240000001</v>
+      </c>
+      <c r="C9">
+        <f>A9*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A9</f>
+        <v>724.72950000000026</v>
+      </c>
+      <c r="D9" s="4">
         <f t="shared" si="0"/>
-        <v>6862.5295200000037</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8">
+        <v>8622.5295199999964</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A10">
         <v>6</v>
       </c>
-      <c r="B8">
-        <f>(A8*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A8)*FARMER_RATE</f>
-        <v>33214.642876800011</v>
-      </c>
-      <c r="C8" s="4">
+      <c r="B10">
+        <f>(MIN(C10,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C10-FARMER_HOURS)*TEMP_WORKER_RATE)+(A10*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C10-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A10*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>43774.642876800011</v>
+      </c>
+      <c r="C10">
+        <f>A10*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A10</f>
+        <v>956.64294000000041</v>
+      </c>
+      <c r="D10" s="4">
         <f t="shared" si="0"/>
-        <v>8052.0346368000028</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9">
+        <v>9812.03463680001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A11">
         <v>7</v>
       </c>
-      <c r="B9">
-        <f>(A9*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A9)*FARMER_RATE</f>
-        <v>42625.458358560019</v>
-      </c>
-      <c r="C9" s="4">
+      <c r="B11">
+        <f>(MIN(C11,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C11-FARMER_HOURS)*TEMP_WORKER_RATE)+(A11*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C11-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A11*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>54945.458358560019</v>
+      </c>
+      <c r="C11">
+        <f>A11*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A11</f>
+        <v>1227.6917730000007</v>
+      </c>
+      <c r="D11" s="4">
         <f t="shared" si="0"/>
-        <v>9410.815481760008</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10">
+        <v>11170.815481760008</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>8</v>
       </c>
-      <c r="B10">
-        <f>(A10*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A10)*FARMER_RATE</f>
-        <v>53586.290507904028</v>
-      </c>
-      <c r="C10" s="4">
+      <c r="B12">
+        <f>(MIN(C12,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C12-FARMER_HOURS)*TEMP_WORKER_RATE)+(A12*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C12-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A12*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>67666.290507904021</v>
+      </c>
+      <c r="C12">
+        <f>A12*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A12</f>
+        <v>1543.3839432000009</v>
+      </c>
+      <c r="D12" s="4">
         <f t="shared" si="0"/>
-        <v>10960.832149344009</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11">
+        <v>12720.832149344002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A13">
         <v>9</v>
       </c>
-      <c r="B11">
-        <f>(A11*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A11)*FARMER_RATE</f>
-        <v>66313.034503531235</v>
-      </c>
-      <c r="C11" s="4">
+      <c r="B13">
+        <f>(MIN(C13,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C13-FARMER_HOURS)*TEMP_WORKER_RATE)+(A13*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C13-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A13*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>82153.034503531235</v>
+      </c>
+      <c r="C13">
+        <f>A13*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A13</f>
+        <v>1909.9376297100011</v>
+      </c>
+      <c r="D13" s="4">
         <f t="shared" si="0"/>
-        <v>12726.743995627206</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12">
+        <v>14486.743995627214</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A14">
         <v>10</v>
       </c>
-      <c r="B12">
-        <f>(A12*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A12)*FARMER_RATE</f>
-        <v>81049.264393204867</v>
-      </c>
-      <c r="C12" s="4">
+      <c r="B14">
+        <f>(MIN(C14,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C14-FARMER_HOURS)*TEMP_WORKER_RATE)+(A14*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C14-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A14*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>98649.264393204867</v>
+      </c>
+      <c r="C14">
+        <f>A14*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A14</f>
+        <v>2334.3682140900019</v>
+      </c>
+      <c r="D14" s="4">
         <f t="shared" si="0"/>
-        <v>14736.229889673632</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A13">
+        <v>16496.229889673632</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A15">
         <v>11</v>
       </c>
-      <c r="B13">
-        <f>(A13*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A13)*FARMER_RATE</f>
-        <v>98069.609915777881</v>
-      </c>
-      <c r="C13" s="4">
+      <c r="B15">
+        <f>(MIN(C15,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C15-FARMER_HOURS)*TEMP_WORKER_RATE)+(A15*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C15-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A15*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>117429.6099157779</v>
+      </c>
+      <c r="C15">
+        <f>A15*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A15</f>
+        <v>2824.5855390489023</v>
+      </c>
+      <c r="D15" s="4">
         <f t="shared" si="0"/>
-        <v>17020.345522573014</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A14">
+        <v>18780.345522573029</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A16">
         <v>12</v>
       </c>
-      <c r="B14">
-        <f>(A14*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A14)*FARMER_RATE</f>
-        <v>117683.53189893346</v>
-      </c>
-      <c r="C14" s="4">
+      <c r="B16">
+        <f>(MIN(C16,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C16-FARMER_HOURS)*TEMP_WORKER_RATE)+(A16*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C16-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A16*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>138803.53189893346</v>
+      </c>
+      <c r="C16">
+        <f>A16*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A16</f>
+        <v>3389.502646858683</v>
+      </c>
+      <c r="D16" s="4">
         <f t="shared" si="0"/>
-        <v>19613.921983155582</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A15">
+        <v>21373.921983155567</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A17">
         <v>13</v>
       </c>
-      <c r="B15">
-        <f>(A15*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A15)*FARMER_RATE</f>
-        <v>140239.54217956238</v>
-      </c>
-      <c r="C15" s="4">
+      <c r="B17">
+        <f>(MIN(C17,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C17-FARMER_HOURS)*TEMP_WORKER_RATE)+(A17*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C17-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A17*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>163119.54217956238</v>
+      </c>
+      <c r="C17">
+        <f>A17*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A17</f>
+        <v>4039.1573208399304</v>
+      </c>
+      <c r="D17" s="4">
         <f t="shared" si="0"/>
-        <v>22556.010280628921</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A16">
+        <v>24316.010280628921</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A18">
         <v>14</v>
       </c>
-      <c r="B16">
-        <f>(A16*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A16)*FARMER_RATE</f>
-        <v>166129.91919732778</v>
-      </c>
-      <c r="C16" s="4">
+      <c r="B18">
+        <f>(MIN(C18,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C18-FARMER_HOURS)*TEMP_WORKER_RATE)+(A18*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C18-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A18*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>190769.91919732775</v>
+      </c>
+      <c r="C18">
+        <f>A18*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A18</f>
+        <v>4784.8479031488414</v>
+      </c>
+      <c r="D18" s="4">
         <f t="shared" si="0"/>
-        <v>25890.377017765393</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A17">
+        <v>27650.377017765364</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A19">
         <v>15</v>
       </c>
-      <c r="B17">
-        <f>(A17*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A17)*FARMER_RATE</f>
-        <v>195795.97619685059</v>
-      </c>
-      <c r="C17" s="4">
+      <c r="B19">
+        <f>(MIN(C19,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C19-FARMER_HOURS)*TEMP_WORKER_RATE)+(A19*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C19-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A19*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>222195.97619685059</v>
+      </c>
+      <c r="C19">
+        <f>A19*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A19</f>
+        <v>5639.2850287111351</v>
+      </c>
+      <c r="D19" s="4">
         <f t="shared" si="0"/>
-        <v>29666.056999522814</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A18">
+        <v>31426.056999522843</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A20">
         <v>16</v>
       </c>
-      <c r="B18">
-        <f>(A18*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A18)*FARMER_RATE</f>
-        <v>229733.94540430469</v>
-      </c>
-      <c r="C18" s="4">
+      <c r="B20">
+        <f>(MIN(C20,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C20-FARMER_HOURS)*TEMP_WORKER_RATE)+(A20*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C20-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A20*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>257893.94540430469</v>
+      </c>
+      <c r="C20">
+        <f>A20*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A20</f>
+        <v>6616.761100354398</v>
+      </c>
+      <c r="D20" s="4">
         <f t="shared" si="0"/>
-        <v>33937.969207454094</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A19">
+        <v>35697.969207454094</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>17</v>
       </c>
-      <c r="B19">
-        <f>(A19*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A19)*FARMER_RATE</f>
-        <v>268501.54869128112</v>
-      </c>
-      <c r="C19" s="4">
+      <c r="B21">
+        <f>(MIN(C21,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C21-FARMER_HOURS)*TEMP_WORKER_RATE)+(A21*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C21-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A21*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>298421.54869128112</v>
+      </c>
+      <c r="C21">
+        <f>A21*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A21</f>
+        <v>7733.3395360392033</v>
+      </c>
+      <c r="D21" s="4">
         <f t="shared" si="0"/>
-        <v>38767.603286976431</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A20">
+        <v>40527.603286976431</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A22">
         <v>18</v>
       </c>
-      <c r="B20">
-        <f>(A20*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A20)*FARMER_RATE</f>
-        <v>312725.33318160975</v>
-      </c>
-      <c r="C20" s="4">
+      <c r="B22">
+        <f>(MIN(C22,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C22-FARMER_HOURS)*TEMP_WORKER_RATE)+(A22*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C22-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A22*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>344405.33318160975</v>
+      </c>
+      <c r="C22">
+        <f>A22*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A22</f>
+        <v>9007.0660478574246</v>
+      </c>
+      <c r="D22" s="4">
         <f t="shared" si="0"/>
-        <v>44223.784490328631</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A21">
+        <v>45983.784490328631</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A23">
         <v>19</v>
       </c>
-      <c r="B21">
-        <f>(A21*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A21)*FARMER_RATE</f>
-        <v>363108.85908309149</v>
-      </c>
-      <c r="C21" s="4">
+      <c r="B23">
+        <f>(MIN(C23,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C23-FARMER_HOURS)*TEMP_WORKER_RATE)+(A23*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C23-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A23*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>396548.85908309149</v>
+      </c>
+      <c r="C23">
+        <f>A23*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A23</f>
+        <v>10458.204466678902</v>
+      </c>
+      <c r="D23" s="4">
         <f t="shared" si="0"/>
-        <v>50383.525901481742</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A22">
+        <v>52143.525901481742</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A24">
         <v>20</v>
       </c>
-      <c r="B22">
-        <f>(A22*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A22)*FARMER_RATE</f>
-        <v>420441.83683305327</v>
-      </c>
-      <c r="C22" s="4">
+      <c r="B24">
+        <f>(MIN(C24,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C24-FARMER_HOURS)*TEMP_WORKER_RATE)+(A24*TOMATO_FERTILIZER_PER_BED)
++(MAX(0,C24-FARMER_HOURS)*TEMP_WORKER_RATE)
++(A24*TOMATO_FERTILIZER_PER_BED)</f>
+        <v>455641.83683305327</v>
+      </c>
+      <c r="C24">
+        <f>A24*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A24</f>
+        <v>12109.499908786096</v>
+      </c>
+      <c r="D24" s="4">
         <f t="shared" si="0"/>
-        <v>57332.977749961778</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="14" t="s">
+        <v>59092.977749961778</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="14" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B25" s="5" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="19"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B28" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C28" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D28" s="5" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>0</v>
+      </c>
+      <c r="B29" s="5">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5">
+        <v>0</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30">
         <v>1</v>
       </c>
-      <c r="B26">
-        <f>(A26*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A26)*FARMER_RATE</f>
-        <v>1067.2129439999999</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="B30">
+        <f>(MIN(C30,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C30-FARMER_HOURS)*TEMP_WORKER_RATE)+(A30*CARROT_FERTILIZER_PER_BED)</f>
+        <v>1507.2129439999999</v>
+      </c>
+      <c r="C30">
+        <f>A30*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A30</f>
+        <v>30.737699999999997</v>
+      </c>
+      <c r="D30" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A27">
+    <row r="31" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A31">
         <v>2</v>
       </c>
-      <c r="B27">
-        <f>(A27*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A27)*FARMER_RATE</f>
-        <v>2187.7865351999994</v>
-      </c>
-      <c r="C27" s="4">
-        <f>B27-B26</f>
-        <v>1120.5735911999996</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A28">
+      <c r="B31">
+        <f>(MIN(C31,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C31-FARMER_HOURS)*TEMP_WORKER_RATE)+(A31*CARROT_FERTILIZER_PER_BED)</f>
+        <v>3067.7865351999994</v>
+      </c>
+      <c r="C31">
+        <f>A31*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A31</f>
+        <v>63.012284999999991</v>
+      </c>
+      <c r="D31" s="4">
+        <f>B31-B30</f>
+        <v>1560.5735911999996</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A32">
         <v>3</v>
       </c>
-      <c r="B28">
-        <f>(A28*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A28)*FARMER_RATE</f>
-        <v>3363.7217978699991</v>
-      </c>
-      <c r="C28" s="4">
-        <f t="shared" ref="C28:C45" si="1">B28-B27</f>
-        <v>1175.9352626699997</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A29">
+      <c r="B32">
+        <f>(MIN(C32,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C32-FARMER_HOURS)*TEMP_WORKER_RATE)+(A32*CARROT_FERTILIZER_PER_BED)</f>
+        <v>4683.7217978699991</v>
+      </c>
+      <c r="C32">
+        <f>A32*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A32</f>
+        <v>96.881388187499979</v>
+      </c>
+      <c r="D32" s="4">
+        <f t="shared" ref="D32:D49" si="1">B32-B31</f>
+        <v>1615.9352626699997</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A33">
         <v>4</v>
       </c>
-      <c r="B29">
-        <f>(A29*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A29)*FARMER_RATE</f>
-        <v>4597.0864570889989</v>
-      </c>
-      <c r="C29" s="4">
+      <c r="B33">
+        <f>(MIN(C33,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C33-FARMER_HOURS)*TEMP_WORKER_RATE)+(A33*CARROT_FERTILIZER_PER_BED)</f>
+        <v>6357.0864570889989</v>
+      </c>
+      <c r="C33">
+        <f>A33*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A33</f>
+        <v>132.40456385624998</v>
+      </c>
+      <c r="D33" s="4">
         <f t="shared" si="1"/>
-        <v>1233.3646592189998</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A30">
+        <v>1673.3646592189998</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A34">
         <v>5</v>
       </c>
-      <c r="B30">
-        <f>(A30*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A30)*FARMER_RATE</f>
-        <v>5890.0170231452794</v>
-      </c>
-      <c r="C30" s="4">
+      <c r="B34">
+        <f>(MIN(C34,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C34-FARMER_HOURS)*TEMP_WORKER_RATE)+(A34*CARROT_FERTILIZER_PER_BED)</f>
+        <v>8090.0170231452794</v>
+      </c>
+      <c r="C34">
+        <f>A34*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A34</f>
+        <v>169.64334744082026</v>
+      </c>
+      <c r="D34" s="4">
         <f t="shared" si="1"/>
-        <v>1292.9305660562804</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A31">
+        <v>1732.9305660562804</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A35">
         <v>6</v>
       </c>
-      <c r="B31">
-        <f>(A31*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A31)*FARMER_RATE</f>
-        <v>7244.7209384686921</v>
-      </c>
-      <c r="C31" s="4">
+      <c r="B35">
+        <f>(MIN(C35,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C35-FARMER_HOURS)*TEMP_WORKER_RATE)+(A35*CARROT_FERTILIZER_PER_BED)</f>
+        <v>9884.7209384686921</v>
+      </c>
+      <c r="C35">
+        <f>A35*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A35</f>
+        <v>208.66131735220887</v>
+      </c>
+      <c r="D35" s="4">
         <f t="shared" si="1"/>
-        <v>1354.7039153234127</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A32">
+        <v>1794.7039153234127</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A36">
         <v>7</v>
       </c>
-      <c r="B32">
-        <f>(A32*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A32)*FARMER_RATE</f>
-        <v>8663.4787889188119</v>
-      </c>
-      <c r="C32" s="4">
+      <c r="B36">
+        <f>(MIN(C36,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C36-FARMER_HOURS)*TEMP_WORKER_RATE)+(A36*CARROT_FERTILIZER_PER_BED)</f>
+        <v>11743.478788918812</v>
+      </c>
+      <c r="C36">
+        <f>A36*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A36</f>
+        <v>249.52415866701648</v>
+      </c>
+      <c r="D36" s="4">
         <f t="shared" si="1"/>
-        <v>1418.7578504501198</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A33">
+        <v>1858.7578504501198</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A37">
         <v>8</v>
       </c>
-      <c r="B33">
-        <f>(A33*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A33)*FARMER_RATE</f>
-        <v>10148.646581304893</v>
-      </c>
-      <c r="C33" s="4">
+      <c r="B37">
+        <f>(MIN(C37,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C37-FARMER_HOURS)*TEMP_WORKER_RATE)+(A37*CARROT_FERTILIZER_PER_BED)</f>
+        <v>13668.646581304893</v>
+      </c>
+      <c r="C37">
+        <f>A37*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A37</f>
+        <v>292.29972872421928</v>
+      </c>
+      <c r="D37" s="4">
         <f t="shared" si="1"/>
-        <v>1485.1677923860807</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A34">
+        <v>1925.1677923860807</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A38">
         <v>9</v>
       </c>
-      <c r="B34">
-        <f>(A34*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A34)*FARMER_RATE</f>
-        <v>11702.658089067203</v>
-      </c>
-      <c r="C34" s="4">
+      <c r="B38">
+        <f>(MIN(C38,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C38-FARMER_HOURS)*TEMP_WORKER_RATE)+(A38*CARROT_FERTILIZER_PER_BED)</f>
+        <v>15662.658089067203</v>
+      </c>
+      <c r="C38">
+        <f>A38*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A38</f>
+        <v>337.05812468511533</v>
+      </c>
+      <c r="D38" s="4">
         <f t="shared" si="1"/>
-        <v>1554.0115077623104</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A35">
+        <v>1994.0115077623104</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A39">
         <v>10</v>
       </c>
-      <c r="B35">
-        <f>(A35*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A35)*FARMER_RATE</f>
-        <v>13328.027268104315</v>
-      </c>
-      <c r="C35" s="4">
+      <c r="B39">
+        <f>(MIN(C39,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C39-FARMER_HOURS)*TEMP_WORKER_RATE)+(A39*CARROT_FERTILIZER_PER_BED)</f>
+        <v>17728.027268104313</v>
+      </c>
+      <c r="C39">
+        <f>A39*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A39</f>
+        <v>383.87175311360357</v>
+      </c>
+      <c r="D39" s="4">
         <f t="shared" si="1"/>
-        <v>1625.3691790371122</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A36">
+        <v>2065.3691790371104</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A40">
         <v>11</v>
       </c>
-      <c r="B36">
-        <f>(A36*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A36)*FARMER_RATE</f>
-        <v>15027.350744787615</v>
-      </c>
-      <c r="C36" s="4">
+      <c r="B40">
+        <f>(MIN(C40,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C40-FARMER_HOURS)*TEMP_WORKER_RATE)+(A40*CARROT_FERTILIZER_PER_BED)</f>
+        <v>19867.350744787615</v>
+      </c>
+      <c r="C40">
+        <f>A40*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A40</f>
+        <v>432.81540163558799</v>
+      </c>
+      <c r="D40" s="4">
         <f t="shared" si="1"/>
-        <v>1699.3234766832993</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A37">
+        <v>2139.3234766833011</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A41">
         <v>12</v>
       </c>
-      <c r="B37">
-        <f>(A37*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A37)*FARMER_RATE</f>
-        <v>16803.310378262511</v>
-      </c>
-      <c r="C37" s="4">
+      <c r="B41">
+        <f>(MIN(C41,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C41-FARMER_HOURS)*TEMP_WORKER_RATE)+(A41*CARROT_FERTILIZER_PER_BED)</f>
+        <v>22083.310378262511</v>
+      </c>
+      <c r="C41">
+        <f>A41*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A41</f>
+        <v>483.96631273797556</v>
+      </c>
+      <c r="D41" s="4">
         <f t="shared" si="1"/>
-        <v>1775.9596334748967</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A38">
+        <v>2215.9596334748967</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A42">
         <v>13</v>
       </c>
-      <c r="B38">
-        <f>(A38*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A38)*FARMER_RATE</f>
-        <v>18658.675899195663</v>
-      </c>
-      <c r="C38" s="4">
+      <c r="B42">
+        <f>(MIN(C42,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C42-FARMER_HOURS)*TEMP_WORKER_RATE)+(A42*CARROT_FERTILIZER_PER_BED)</f>
+        <v>24378.675899195663</v>
+      </c>
+      <c r="C42">
+        <f>A42*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A42</f>
+        <v>537.4042597694604</v>
+      </c>
+      <c r="D42" s="4">
         <f t="shared" si="1"/>
-        <v>1855.3655209331519</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A39">
+        <v>2295.3655209331519</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A43">
         <v>14</v>
       </c>
-      <c r="B39">
-        <f>(A39*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A39)*FARMER_RATE</f>
-        <v>20596.30762718906</v>
-      </c>
-      <c r="C39" s="4">
+      <c r="B43">
+        <f>(MIN(C43,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C43-FARMER_HOURS)*TEMP_WORKER_RATE)+(A43*CARROT_FERTILIZER_PER_BED)</f>
+        <v>26756.30762718906</v>
+      </c>
+      <c r="C43">
+        <f>A43*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A43</f>
+        <v>593.2116252070582</v>
+      </c>
+      <c r="D43" s="4">
         <f t="shared" si="1"/>
-        <v>1937.6317279933974</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A40">
+        <v>2377.6317279933974</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A44">
         <v>15</v>
       </c>
-      <c r="B40">
-        <f>(A40*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A40)*FARMER_RATE</f>
-        <v>22619.15926914513</v>
-      </c>
-      <c r="C40" s="4">
+      <c r="B44">
+        <f>(MIN(C44,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C44-FARMER_HOURS)*TEMP_WORKER_RATE)+(A44*CARROT_FERTILIZER_PER_BED)</f>
+        <v>29219.15926914513</v>
+      </c>
+      <c r="C44">
+        <f>A44*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A44</f>
+        <v>651.47348125418</v>
+      </c>
+      <c r="D44" s="4">
         <f t="shared" si="1"/>
-        <v>2022.8516419560692</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A41">
+        <v>2462.8516419560692</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A45">
         <v>16</v>
       </c>
-      <c r="B41">
-        <f>(A41*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A41)*FARMER_RATE</f>
-        <v>24730.280800932007</v>
-      </c>
-      <c r="C41" s="4">
+      <c r="B45">
+        <f>(MIN(C45,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C45-FARMER_HOURS)*TEMP_WORKER_RATE)+(A45*CARROT_FERTILIZER_PER_BED)</f>
+        <v>31770.280800932007</v>
+      </c>
+      <c r="C45">
+        <f>A45*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A45</f>
+        <v>712.27767283790342</v>
+      </c>
+      <c r="D45" s="4">
         <f t="shared" si="1"/>
-        <v>2111.1215317868773</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A42">
+        <v>2551.1215317868773</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A46">
         <v>17</v>
       </c>
-      <c r="B42">
-        <f>(A42*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A42)*FARMER_RATE</f>
-        <v>26932.82143476501</v>
-      </c>
-      <c r="C42" s="4">
+      <c r="B46">
+        <f>(MIN(C46,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C46-FARMER_HOURS)*TEMP_WORKER_RATE)+(A46*CARROT_FERTILIZER_PER_BED)</f>
+        <v>33445.6107173825</v>
+      </c>
+      <c r="C46">
+        <f>A46*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A46</f>
+        <v>775.71490307502916</v>
+      </c>
+      <c r="D46" s="4">
         <f t="shared" si="1"/>
-        <v>2202.5406338330031</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A43">
+        <v>1675.3299164504933</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A47">
         <v>18</v>
       </c>
-      <c r="B43">
-        <f>(A43*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A43)*FARMER_RATE</f>
-        <v>29230.032674789087</v>
-      </c>
-      <c r="C43" s="4">
+      <c r="B47">
+        <f>(MIN(C47,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C47-FARMER_HOURS)*TEMP_WORKER_RATE)+(A47*CARROT_FERTILIZER_PER_BED)</f>
+        <v>35034.216337394537</v>
+      </c>
+      <c r="C47">
+        <f>A47*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A47</f>
+        <v>841.87882127848752</v>
+      </c>
+      <c r="D47" s="4">
         <f t="shared" si="1"/>
-        <v>2297.2112400240767</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A44">
+        <v>1588.6056200120365</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A48">
         <v>19</v>
       </c>
-      <c r="B44">
-        <f>(A44*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A44)*FARMER_RATE</f>
-        <v>31625.271463417637</v>
-      </c>
-      <c r="C44" s="4">
+      <c r="B48">
+        <f>(MIN(C48,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C48-FARMER_HOURS)*TEMP_WORKER_RATE)+(A48*CARROT_FERTILIZER_PER_BED)</f>
+        <v>36671.835731708816</v>
+      </c>
+      <c r="C48">
+        <f>A48*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A48</f>
+        <v>910.86611357769698</v>
+      </c>
+      <c r="D48" s="4">
         <f t="shared" si="1"/>
-        <v>2395.2387886285505</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A45">
+        <v>1637.6193943142789</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A49">
         <v>20</v>
       </c>
-      <c r="B45">
-        <f>(A45*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A45)*FARMER_RATE</f>
-        <v>34122.003421055866</v>
-      </c>
-      <c r="C45" s="4">
+      <c r="B49">
+        <f>(MIN(C49,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C49-FARMER_HOURS)*TEMP_WORKER_RATE)+(A49*CARROT_FERTILIZER_PER_BED)</f>
+        <v>38360.20171052793</v>
+      </c>
+      <c r="C49">
+        <f>A49*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A49</f>
+        <v>982.77659622856766</v>
+      </c>
+      <c r="D49" s="4">
         <f t="shared" si="1"/>
-        <v>2496.7319576382288</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A47" s="15" t="s">
+        <v>1688.3659788191144</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A51" s="15" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A48" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="B48" s="5" t="s">
+    <row r="52" spans="1:4" s="17" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A52" s="16"/>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="B53" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="C48" s="5" t="s">
+      <c r="C53" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D53" s="5" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="18">
+        <v>0</v>
+      </c>
+      <c r="B54" s="5">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5">
+        <v>0</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A55">
         <v>1</v>
       </c>
-      <c r="B49">
-        <f>((A49*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A49)*FARMER_RATE)
-+(A49*MESCLUN_FERTILIZER_PER_BED)</f>
+      <c r="B55">
+        <f>(MIN(C55,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C55-FARMER_HOURS)*TEMP_WORKER_RATE)+(A55*MESCLUN_FERTILIZER_PER_BED)</f>
         <v>2461.9299999999998</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C55" s="4">
+        <f>A55*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A55</f>
+        <v>45.5625</v>
+      </c>
+      <c r="D55" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A50">
+    <row r="56" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A56">
         <v>2</v>
       </c>
-      <c r="B50">
-        <f>((A50*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A50)*FARMER_RATE)
-+(A50*MESCLUN_FERTILIZER_PER_BED)</f>
+      <c r="B56">
+        <f>(MIN(C56,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C56-FARMER_HOURS)*TEMP_WORKER_RATE)+(A56*MESCLUN_FERTILIZER_PER_BED)</f>
         <v>4963.4082499999995</v>
       </c>
-      <c r="C50" s="4">
-        <f>B50-B49</f>
+      <c r="C56" s="4">
+        <f>A56*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A56</f>
+        <v>92.264062499999994</v>
+      </c>
+      <c r="D56" s="4">
+        <f>B56-B55</f>
         <v>2501.4782499999997</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A51">
+    <row r="57" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A57">
         <v>3</v>
       </c>
-      <c r="B51">
-        <f>((A51*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A51)*FARMER_RATE)
-+(A51*MESCLUN_FERTILIZER_PER_BED)</f>
+      <c r="B57">
+        <f>(MIN(C57,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C57-FARMER_HOURS)*TEMP_WORKER_RATE)+(A57*MESCLUN_FERTILIZER_PER_BED)</f>
         <v>7505.1762796874991</v>
       </c>
-      <c r="C51" s="4">
-        <f t="shared" ref="C51:C78" si="2">B51-B50</f>
+      <c r="C57" s="4">
+        <f>A57*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A57</f>
+        <v>140.12604492187498</v>
+      </c>
+      <c r="D57" s="4">
+        <f t="shared" ref="D57:D84" si="2">B57-B56</f>
         <v>2541.7680296874996</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A52">
+    <row r="58" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A58">
         <v>4</v>
       </c>
-      <c r="B52">
-        <f>((A52*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A52)*FARMER_RATE)
-+(A52*MESCLUN_FERTILIZER_PER_BED)</f>
+      <c r="B58">
+        <f>(MIN(C58,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C58-FARMER_HOURS)*TEMP_WORKER_RATE)+(A58*MESCLUN_FERTILIZER_PER_BED)</f>
         <v>10087.987977578125</v>
       </c>
-      <c r="C52" s="4">
+      <c r="C58" s="4">
+        <f>A58*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A58</f>
+        <v>189.17016064453125</v>
+      </c>
+      <c r="D58" s="4">
         <f t="shared" si="2"/>
         <v>2582.8116978906255</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A53">
+    <row r="59" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A59">
         <v>5</v>
       </c>
-      <c r="B53">
-        <f>((A53*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A53)*FARMER_RATE)
-+(A53*MESCLUN_FERTILIZER_PER_BED)</f>
+      <c r="B59">
+        <f>(MIN(C59,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C59-FARMER_HOURS)*TEMP_WORKER_RATE)+(A59*MESCLUN_FERTILIZER_PER_BED)</f>
         <v>12712.609784122313</v>
       </c>
-      <c r="C53" s="4">
+      <c r="C59" s="4">
+        <f>A59*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A59</f>
+        <v>239.41848456573481</v>
+      </c>
+      <c r="D59" s="4">
         <f t="shared" si="2"/>
         <v>2624.6218065441881</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A54">
+    <row r="60" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A60">
         <v>6</v>
       </c>
-      <c r="B54">
-        <f>((A54*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A54)*FARMER_RATE)
-+(A54*MESCLUN_FERTILIZER_PER_BED)</f>
+      <c r="B60">
+        <f>(MIN(C60,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C60-FARMER_HOURS)*TEMP_WORKER_RATE)+(A60*MESCLUN_FERTILIZER_PER_BED)</f>
         <v>15379.820887708611</v>
       </c>
-      <c r="C54" s="4">
+      <c r="C60" s="4">
+        <f>A60*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A60</f>
+        <v>290.89345874736784</v>
+      </c>
+      <c r="D60" s="4">
         <f t="shared" si="2"/>
         <v>2667.2111035862981</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A55">
+    <row r="61" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A61">
         <v>7</v>
       </c>
-      <c r="B55">
-        <f>((A55*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A55)*FARMER_RATE)
-+(A55*MESCLUN_FERTILIZER_PER_BED)</f>
+      <c r="B61">
+        <f>(MIN(C61,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C61-FARMER_HOURS)*TEMP_WORKER_RATE)+(A61*MESCLUN_FERTILIZER_PER_BED)</f>
         <v>18090.413423605794</v>
       </c>
-      <c r="C55" s="4">
+      <c r="C61" s="4">
+        <f>A61*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A61</f>
+        <v>343.61789814532818</v>
+      </c>
+      <c r="D61" s="4">
         <f t="shared" si="2"/>
         <v>2710.5925358971836</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A56">
+    <row r="62" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A62">
         <v>8</v>
       </c>
-      <c r="B56">
-        <f>((A56*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A56)*FARMER_RATE)
-+(A56*MESCLUN_FERTILIZER_PER_BED)</f>
+      <c r="B62">
+        <f>(MIN(C62,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C62-FARMER_HOURS)*TEMP_WORKER_RATE)+(A62*MESCLUN_FERTILIZER_PER_BED)</f>
         <v>20845.192675886705</v>
       </c>
-      <c r="C56" s="4">
+      <c r="C62" s="4">
+        <f>A62*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A62</f>
+        <v>397.61499642530839</v>
+      </c>
+      <c r="D62" s="4">
         <f t="shared" si="2"/>
         <v>2754.7792522809104</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A57">
+    <row r="63" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A63">
         <v>9</v>
       </c>
-      <c r="B57">
-        <f>((A57*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A57)*FARMER_RATE)
-+(A57*MESCLUN_FERTILIZER_PER_BED)</f>
+      <c r="B63">
+        <f>(MIN(C63,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C63-FARMER_HOURS)*TEMP_WORKER_RATE)+(A63*MESCLUN_FERTILIZER_PER_BED)</f>
         <v>23644.9772823772</v>
       </c>
-      <c r="C57" s="4">
+      <c r="C63" s="4">
+        <f>A63*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A63</f>
+        <v>452.90833186570285</v>
+      </c>
+      <c r="D63" s="4">
         <f t="shared" si="2"/>
         <v>2799.7846064904952</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A58">
+    <row r="64" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A64">
         <v>10</v>
       </c>
-      <c r="B58">
-        <f>((A58*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A58)*FARMER_RATE)
-+(A58*MESCLUN_FERTILIZER_PER_BED)</f>
+      <c r="B64">
+        <f>(MIN(C64,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C64-FARMER_HOURS)*TEMP_WORKER_RATE)+(A64*MESCLUN_FERTILIZER_PER_BED)</f>
         <v>26490.599442674353</v>
       </c>
-      <c r="C58" s="4">
+      <c r="C64" s="4">
+        <f>A64*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A64</f>
+        <v>509.52187334891573</v>
+      </c>
+      <c r="D64" s="4">
         <f t="shared" si="2"/>
         <v>2845.6221602971527</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A59">
+    <row r="65" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A65">
         <v>11</v>
       </c>
-      <c r="B59">
-        <f>((A59*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A59)*FARMER_RATE)
-+(A59*MESCLUN_FERTILIZER_PER_BED)</f>
+      <c r="B65">
+        <f>(MIN(C65,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C65-FARMER_HOURS)*TEMP_WORKER_RATE)+(A65*MESCLUN_FERTILIZER_PER_BED)</f>
         <v>29382.905129278555</v>
       </c>
-      <c r="C59" s="4">
+      <c r="C65" s="4">
+        <f>A65*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A65</f>
+        <v>567.47998644235474</v>
+      </c>
+      <c r="D65" s="4">
         <f t="shared" si="2"/>
         <v>2892.3056866042025</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A60">
+    <row r="66" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A66">
         <v>12</v>
       </c>
-      <c r="B60">
-        <f>((A60*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A60)*FARMER_RATE)
-+(A60*MESCLUN_FERTILIZER_PER_BED)</f>
+      <c r="B66">
+        <f>(MIN(C66,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C66-FARMER_HOURS)*TEMP_WORKER_RATE)+(A66*MESCLUN_FERTILIZER_PER_BED)</f>
         <v>32322.754301884954</v>
       </c>
-      <c r="C60" s="4">
+      <c r="C66" s="4">
+        <f>A66*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A66</f>
+        <v>626.80743957041921</v>
+      </c>
+      <c r="D66" s="4">
         <f t="shared" si="2"/>
         <v>2939.8491726063985</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A61">
+    <row r="67" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A67">
         <v>13</v>
       </c>
-      <c r="B61">
-        <f>((A61*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A61)*FARMER_RATE)
-+(A61*MESCLUN_FERTILIZER_PER_BED)</f>
+      <c r="B67">
+        <f>(MIN(C67,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C67-FARMER_HOURS)*TEMP_WORKER_RATE)+(A67*MESCLUN_FERTILIZER_PER_BED)</f>
         <v>35311.021124880055</v>
       </c>
-      <c r="C61" s="4">
+      <c r="C67" s="4">
+        <f>A67*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A67</f>
+        <v>687.52941027880343</v>
+      </c>
+      <c r="D67" s="4">
         <f t="shared" si="2"/>
         <v>2988.2668229951014</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A62">
+    <row r="68" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A68">
         <v>14</v>
       </c>
-      <c r="B62">
-        <f>((A62*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A62)*FARMER_RATE)
-+(A62*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>38348.59418809037</v>
-      </c>
-      <c r="C62" s="4">
+      <c r="B68">
+        <f>(MIN(C68,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C68-FARMER_HOURS)*TEMP_WORKER_RATE)+(A68*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>37833.497094045189</v>
+      </c>
+      <c r="C68" s="4">
+        <f>A68*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A68</f>
+        <v>749.67149159246469</v>
+      </c>
+      <c r="D68" s="4">
         <f t="shared" si="2"/>
-        <v>3037.573063210315</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A63">
+        <v>2522.4759691651343</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A69">
         <v>15</v>
       </c>
-      <c r="B63">
-        <f>((A63*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A63)*FARMER_RATE)
-+(A63*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>41436.376730830176</v>
-      </c>
-      <c r="C63" s="4">
+      <c r="B69">
+        <f>(MIN(C69,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C69-FARMER_HOURS)*TEMP_WORKER_RATE)+(A69*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>39817.388365415085</v>
+      </c>
+      <c r="C69" s="4">
+        <f>A69*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A69</f>
+        <v>813.25969846861108</v>
+      </c>
+      <c r="D69" s="4">
         <f t="shared" si="2"/>
-        <v>3087.7825427398056</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A64">
+        <v>1983.8912713698955</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A70">
         <v>16</v>
       </c>
-      <c r="B64">
-        <f>((A64*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A64)*FARMER_RATE)
-+(A64*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>44575.2868692966</v>
-      </c>
-      <c r="C64" s="4">
+      <c r="B70">
+        <f>(MIN(C70,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C70-FARMER_HOURS)*TEMP_WORKER_RATE)+(A70*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>41826.843434648297</v>
+      </c>
+      <c r="C70" s="4">
+        <f>A70*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A70</f>
+        <v>878.32047434610013</v>
+      </c>
+      <c r="D70" s="4">
         <f t="shared" si="2"/>
-        <v>3138.9101384664245</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A65">
+        <v>2009.4550692332123</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A71">
         <v>17</v>
       </c>
-      <c r="B65">
-        <f>((A65*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A65)*FARMER_RATE)
-+(A65*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>47766.257827360474</v>
-      </c>
-      <c r="C65" s="4">
+      <c r="B71">
+        <f>(MIN(C71,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C71-FARMER_HOURS)*TEMP_WORKER_RATE)+(A71*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>43862.328913680234</v>
+      </c>
+      <c r="C71" s="4">
+        <f>A71*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A71</f>
+        <v>944.88069779264049</v>
+      </c>
+      <c r="D71" s="4">
         <f t="shared" si="2"/>
-        <v>3190.9709580638737</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A66">
+        <v>2035.4854790319368</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A72">
         <v>18</v>
       </c>
-      <c r="B66">
-        <f>((A66*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A66)*FARMER_RATE)
-+(A66*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>51010.23817080263</v>
-      </c>
-      <c r="C66" s="4">
+      <c r="B72">
+        <f>(MIN(C72,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C72-FARMER_HOURS)*TEMP_WORKER_RATE)+(A72*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>45924.319085401308</v>
+      </c>
+      <c r="C72" s="4">
+        <f>A72*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A72</f>
+        <v>1012.9676892512279</v>
+      </c>
+      <c r="D72" s="4">
         <f t="shared" si="2"/>
-        <v>3243.9803434421556</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A67">
+        <v>2061.9901717210741</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A73">
         <v>19</v>
       </c>
-      <c r="B67">
-        <f>((A67*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A67)*FARMER_RATE)
-+(A67*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>54308.192045045304</v>
-      </c>
-      <c r="C67" s="4">
+      <c r="B73">
+        <f>(MIN(C73,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C73-FARMER_HOURS)*TEMP_WORKER_RATE)+(A73*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>48013.296022522649</v>
+      </c>
+      <c r="C73" s="4">
+        <f>A73*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A73</f>
+        <v>1082.6092178872495</v>
+      </c>
+      <c r="D73" s="4">
         <f t="shared" si="2"/>
-        <v>3297.9538742426739</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A68">
+        <v>2088.9769371213406</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A74">
         <v>20</v>
       </c>
-      <c r="B68">
-        <f>((A68*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A68)*FARMER_RATE)
-+(A68*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>57661.099416429868</v>
-      </c>
-      <c r="C68" s="4">
+      <c r="B74">
+        <f>(MIN(C74,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C74-FARMER_HOURS)*TEMP_WORKER_RATE)+(A74*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>50129.749708214935</v>
+      </c>
+      <c r="C74" s="4">
+        <f>A74*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A74</f>
+        <v>1153.8335085377266</v>
+      </c>
+      <c r="D74" s="4">
         <f t="shared" si="2"/>
-        <v>3352.9073713845646</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A69">
+        <v>2116.4536856922859</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A75">
         <v>21</v>
       </c>
-      <c r="B69">
-        <f>((A69*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A69)*FARMER_RATE)
-+(A69*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>61069.956317091994</v>
-      </c>
-      <c r="C69" s="4">
+      <c r="B75">
+        <f>(MIN(C75,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C75-FARMER_HOURS)*TEMP_WORKER_RATE)+(A75*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>52274.178158545998</v>
+      </c>
+      <c r="C75" s="4">
+        <f>A75*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A75</f>
+        <v>1226.6692487641703</v>
+      </c>
+      <c r="D75" s="4">
         <f t="shared" si="2"/>
-        <v>3408.8569006621256</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A70">
+        <v>2144.4284503310628</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A76">
         <v>22</v>
       </c>
-      <c r="B70">
-        <f>((A70*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A70)*FARMER_RATE)
-+(A70*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>64535.775093486867</v>
-      </c>
-      <c r="C70" s="4">
+      <c r="B76">
+        <f>(MIN(C76,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C76-FARMER_HOURS)*TEMP_WORKER_RATE)+(A76*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>54447.087546743431</v>
+      </c>
+      <c r="C76" s="4">
+        <f>A76*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A76</f>
+        <v>1301.1455960105666</v>
+      </c>
+      <c r="D76" s="4">
         <f t="shared" si="2"/>
-        <v>3465.8187763948736</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A71">
+        <v>2172.9093881974331</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A77">
         <v>23</v>
       </c>
-      <c r="B71">
-        <f>((A71*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A71)*FARMER_RATE)
-+(A71*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>68059.584658617066</v>
-      </c>
-      <c r="C71" s="4">
+      <c r="B77">
+        <f>(MIN(C77,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C77-FARMER_HOURS)*TEMP_WORKER_RATE)+(A77*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>56648.99232930853</v>
+      </c>
+      <c r="C77" s="4">
+        <f>A77*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A77</f>
+        <v>1377.292184868003</v>
+      </c>
+      <c r="D77" s="4">
         <f t="shared" si="2"/>
-        <v>3523.8095651301992</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A72">
+        <v>2201.9047825650996</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A78">
         <v>24</v>
       </c>
-      <c r="B72">
-        <f>((A72*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A72)*FARMER_RATE)
-+(A72*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>71642.430748017156</v>
-      </c>
-      <c r="C72" s="4">
+      <c r="B78">
+        <f>(MIN(C78,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C78-FARMER_HOURS)*TEMP_WORKER_RATE)+(A78*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>58880.415374008575</v>
+      </c>
+      <c r="C78" s="4">
+        <f>A78*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A78</f>
+        <v>1455.1391344474989</v>
+      </c>
+      <c r="D78" s="4">
         <f t="shared" si="2"/>
-        <v>3582.8460894000891</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A73">
+        <v>2231.4230447000446</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A79">
         <v>25</v>
       </c>
-      <c r="B73">
-        <f>((A73*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A73)*FARMER_RATE)
-+(A73*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>75285.376179549348</v>
-      </c>
-      <c r="C73" s="4">
+      <c r="B79">
+        <f>(MIN(C79,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C79-FARMER_HOURS)*TEMP_WORKER_RATE)+(A79*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>61141.888089774671</v>
+      </c>
+      <c r="C79" s="4">
+        <f>A79*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A79</f>
+        <v>1534.7170558625965</v>
+      </c>
+      <c r="D79" s="4">
         <f t="shared" si="2"/>
-        <v>3642.9454315321927</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A74">
+        <v>2261.4727157660964</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A80">
         <v>26</v>
       </c>
-      <c r="B74">
-        <f>((A74*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A74)*FARMER_RATE)
-+(A74*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>78989.501117065476</v>
-      </c>
-      <c r="C74" s="4">
+      <c r="B80">
+        <f>(MIN(C80,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C80-FARMER_HOURS)*TEMP_WORKER_RATE)+(A80*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>63433.950558532735</v>
+      </c>
+      <c r="C80" s="4">
+        <f>A80*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A80</f>
+        <v>1616.0570598233144</v>
+      </c>
+      <c r="D80" s="4">
         <f t="shared" si="2"/>
-        <v>3704.1249375161278</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A75">
+        <v>2292.0624687580639</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A81">
         <v>27</v>
       </c>
-      <c r="B75">
-        <f>((A75*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A75)*FARMER_RATE)
-+(A75*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>82755.903337991418</v>
-      </c>
-      <c r="C75" s="4">
+      <c r="B81">
+        <f>(MIN(C81,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C81-FARMER_HOURS)*TEMP_WORKER_RATE)+(A81*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>65757.151668995706</v>
+      </c>
+      <c r="C81" s="4">
+        <f>A81*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A81</f>
+        <v>1699.1907643430709</v>
+      </c>
+      <c r="D81" s="4">
         <f t="shared" si="2"/>
-        <v>3766.4022209259419</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A76">
+        <v>2323.201110462971</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A82">
         <v>28</v>
       </c>
-      <c r="B76">
-        <f>((A76*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A76)*FARMER_RATE)
-+(A76*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>86585.698504890999</v>
-      </c>
-      <c r="C76" s="4">
+      <c r="B82">
+        <f>(MIN(C82,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C82-FARMER_HOURS)*TEMP_WORKER_RATE)+(A82*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>68112.049252445489</v>
+      </c>
+      <c r="C82" s="4">
+        <f>A82*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A82</f>
+        <v>1784.1503025602246</v>
+      </c>
+      <c r="D82" s="4">
         <f t="shared" si="2"/>
-        <v>3829.7951668995811</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A77">
+        <v>2354.8975834497833</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A83">
         <v>29</v>
       </c>
-      <c r="B77">
-        <f>((A77*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A77)*FARMER_RATE)
-+(A77*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>90480.020441066488</v>
-      </c>
-      <c r="C77" s="4">
+      <c r="B83">
+        <f>(MIN(C83,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C83-FARMER_HOURS)*TEMP_WORKER_RATE)+(A83*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>70499.210220533249</v>
+      </c>
+      <c r="C83" s="4">
+        <f>A83*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A83</f>
+        <v>1870.9683306758782</v>
+      </c>
+      <c r="D83" s="4">
         <f t="shared" si="2"/>
-        <v>3894.3219361754891</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A78">
+        <v>2387.1609680877591</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A84">
         <v>30</v>
       </c>
-      <c r="B78">
-        <f>((A78*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A78)*FARMER_RATE)
-+(A78*MESCLUN_FERTILIZER_PER_BED)</f>
-        <v>94440.021410255009</v>
-      </c>
-      <c r="C78" s="4">
+      <c r="B84">
+        <f>(MIN(C84,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C84-FARMER_HOURS)*TEMP_WORKER_RATE)+(A84*MESCLUN_FERTILIZER_PER_BED)</f>
+        <v>72919.210705127509</v>
+      </c>
+      <c r="C84" s="4">
+        <f>A84*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A84</f>
+        <v>1959.6780360096488</v>
+      </c>
+      <c r="D84" s="4">
         <f t="shared" si="2"/>
-        <v>3960.0009691885207</v>
+        <v>2420.0004845942603</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated values on Checks worksheet
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6fd52bb83a98f88c/Desktop/BUS 620 Economics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2068" documentId="8_{202E0E92-0A53-4DF2-844D-22EFC22CE560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04736648-7896-4C13-B99A-77F5A00D15DE}"/>
+  <xr:revisionPtr revIDLastSave="2073" documentId="8_{202E0E92-0A53-4DF2-844D-22EFC22CE560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{453CF89E-C8E5-43C1-BA7E-B90288FDAF88}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="450" windowWidth="22935" windowHeight="13935" firstSheet="5" activeTab="7" xr2:uid="{CB3B63E6-161E-4EB6-9C62-E77ECB56D41C}"/>
+    <workbookView xWindow="0" yWindow="450" windowWidth="22935" windowHeight="13935" activeTab="3" xr2:uid="{CB3B63E6-161E-4EB6-9C62-E77ECB56D41C}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="8" r:id="rId1"/>
@@ -686,7 +686,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -721,15 +721,11 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1627,7 +1623,7 @@
         <v>20</v>
       </c>
       <c r="B24">
-        <f>B13-B18-B22-20000</f>
+        <f>B13-B18-B22-FIXED_COSTS</f>
         <v>42775.155387742139</v>
       </c>
     </row>
@@ -1729,7 +1725,8 @@
         <v>23</v>
       </c>
       <c r="B2">
-        <v>99</v>
+        <f>1*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)</f>
+        <v>99.000000000000014</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
@@ -1737,7 +1734,7 @@
         <v>24</v>
       </c>
       <c r="B3" s="4">
-        <f>1*2.5*36*1.1</f>
+        <f>1*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)</f>
         <v>99.000000000000014</v>
       </c>
     </row>
@@ -2965,13 +2962,13 @@
         <v>1</v>
       </c>
       <c r="B5">
-        <f>(MIN(C5,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C5-FARMER_HOURS)*TEMP_WORKER_RATE)+(A5*TOMATO_FERTILIZER_PER_BED)
+        <f t="shared" ref="B5:B24" si="0">(MIN(C5,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C5-FARMER_HOURS)*TEMP_WORKER_RATE)+(A5*TOMATO_FERTILIZER_PER_BED)
 +(MAX(0,C5-FARMER_HOURS)*TEMP_WORKER_RATE)
 +(A5*TOMATO_FERTILIZER_PER_BED)</f>
         <v>5197.2800000000007</v>
       </c>
       <c r="C5">
-        <f>A5*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A5</f>
+        <f t="shared" ref="C5:C24" si="1">A5*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A5</f>
         <v>99.000000000000014</v>
       </c>
       <c r="D5" t="s">
@@ -2983,13 +2980,11 @@
         <v>2</v>
       </c>
       <c r="B6">
-        <f>(MIN(C6,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C6-FARMER_HOURS)*TEMP_WORKER_RATE)+(A6*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C6-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A6*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>11082.016000000001</v>
       </c>
       <c r="C6">
-        <f>A6*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A6</f>
+        <f t="shared" si="1"/>
         <v>217.80000000000004</v>
       </c>
       <c r="D6" s="4">
@@ -3002,17 +2997,15 @@
         <v>3</v>
       </c>
       <c r="B7">
-        <f>(MIN(C7,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C7-FARMER_HOURS)*TEMP_WORKER_RATE)+(A7*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C7-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A7*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>17757.326400000005</v>
       </c>
       <c r="C7">
-        <f>A7*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A7</f>
+        <f t="shared" si="1"/>
         <v>359.37000000000012</v>
       </c>
       <c r="D7" s="4">
-        <f t="shared" ref="D7:D24" si="0">B7-B6</f>
+        <f t="shared" ref="D7:D24" si="2">B7-B6</f>
         <v>6675.3104000000039</v>
       </c>
     </row>
@@ -3021,17 +3014,15 @@
         <v>4</v>
       </c>
       <c r="B8">
-        <f>(MIN(C8,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C8-FARMER_HOURS)*TEMP_WORKER_RATE)+(A8*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C8-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A8*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>25340.078720000005</v>
       </c>
       <c r="C8">
-        <f>A8*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A8</f>
+        <f t="shared" si="1"/>
         <v>527.07600000000014</v>
       </c>
       <c r="D8" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>7582.7523199999996</v>
       </c>
     </row>
@@ -3040,17 +3031,15 @@
         <v>5</v>
       </c>
       <c r="B9">
-        <f>(MIN(C9,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C9-FARMER_HOURS)*TEMP_WORKER_RATE)+(A9*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C9-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A9*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>33962.608240000001</v>
       </c>
       <c r="C9">
-        <f>A9*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A9</f>
+        <f t="shared" si="1"/>
         <v>724.72950000000026</v>
       </c>
       <c r="D9" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>8622.5295199999964</v>
       </c>
     </row>
@@ -3059,17 +3048,15 @@
         <v>6</v>
       </c>
       <c r="B10">
-        <f>(MIN(C10,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C10-FARMER_HOURS)*TEMP_WORKER_RATE)+(A10*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C10-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A10*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>43774.642876800011</v>
       </c>
       <c r="C10">
-        <f>A10*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A10</f>
+        <f t="shared" si="1"/>
         <v>956.64294000000041</v>
       </c>
       <c r="D10" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>9812.03463680001</v>
       </c>
     </row>
@@ -3078,17 +3065,15 @@
         <v>7</v>
       </c>
       <c r="B11">
-        <f>(MIN(C11,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C11-FARMER_HOURS)*TEMP_WORKER_RATE)+(A11*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C11-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A11*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>54945.458358560019</v>
       </c>
       <c r="C11">
-        <f>A11*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A11</f>
+        <f t="shared" si="1"/>
         <v>1227.6917730000007</v>
       </c>
       <c r="D11" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>11170.815481760008</v>
       </c>
     </row>
@@ -3097,17 +3082,15 @@
         <v>8</v>
       </c>
       <c r="B12">
-        <f>(MIN(C12,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C12-FARMER_HOURS)*TEMP_WORKER_RATE)+(A12*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C12-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A12*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>67666.290507904021</v>
       </c>
       <c r="C12">
-        <f>A12*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A12</f>
+        <f t="shared" si="1"/>
         <v>1543.3839432000009</v>
       </c>
       <c r="D12" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>12720.832149344002</v>
       </c>
     </row>
@@ -3116,17 +3099,15 @@
         <v>9</v>
       </c>
       <c r="B13">
-        <f>(MIN(C13,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C13-FARMER_HOURS)*TEMP_WORKER_RATE)+(A13*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C13-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A13*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>82153.034503531235</v>
       </c>
       <c r="C13">
-        <f>A13*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A13</f>
+        <f t="shared" si="1"/>
         <v>1909.9376297100011</v>
       </c>
       <c r="D13" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>14486.743995627214</v>
       </c>
     </row>
@@ -3135,17 +3116,15 @@
         <v>10</v>
       </c>
       <c r="B14">
-        <f>(MIN(C14,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C14-FARMER_HOURS)*TEMP_WORKER_RATE)+(A14*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C14-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A14*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>98649.264393204867</v>
       </c>
       <c r="C14">
-        <f>A14*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A14</f>
+        <f t="shared" si="1"/>
         <v>2334.3682140900019</v>
       </c>
       <c r="D14" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>16496.229889673632</v>
       </c>
     </row>
@@ -3154,17 +3133,15 @@
         <v>11</v>
       </c>
       <c r="B15">
-        <f>(MIN(C15,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C15-FARMER_HOURS)*TEMP_WORKER_RATE)+(A15*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C15-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A15*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>117429.6099157779</v>
       </c>
       <c r="C15">
-        <f>A15*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A15</f>
+        <f t="shared" si="1"/>
         <v>2824.5855390489023</v>
       </c>
       <c r="D15" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>18780.345522573029</v>
       </c>
     </row>
@@ -3173,17 +3150,15 @@
         <v>12</v>
       </c>
       <c r="B16">
-        <f>(MIN(C16,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C16-FARMER_HOURS)*TEMP_WORKER_RATE)+(A16*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C16-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A16*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>138803.53189893346</v>
       </c>
       <c r="C16">
-        <f>A16*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A16</f>
+        <f t="shared" si="1"/>
         <v>3389.502646858683</v>
       </c>
       <c r="D16" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>21373.921983155567</v>
       </c>
     </row>
@@ -3192,17 +3167,15 @@
         <v>13</v>
       </c>
       <c r="B17">
-        <f>(MIN(C17,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C17-FARMER_HOURS)*TEMP_WORKER_RATE)+(A17*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C17-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A17*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>163119.54217956238</v>
       </c>
       <c r="C17">
-        <f>A17*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A17</f>
+        <f t="shared" si="1"/>
         <v>4039.1573208399304</v>
       </c>
       <c r="D17" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>24316.010280628921</v>
       </c>
     </row>
@@ -3211,17 +3184,15 @@
         <v>14</v>
       </c>
       <c r="B18">
-        <f>(MIN(C18,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C18-FARMER_HOURS)*TEMP_WORKER_RATE)+(A18*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C18-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A18*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>190769.91919732775</v>
       </c>
       <c r="C18">
-        <f>A18*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A18</f>
+        <f t="shared" si="1"/>
         <v>4784.8479031488414</v>
       </c>
       <c r="D18" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>27650.377017765364</v>
       </c>
     </row>
@@ -3230,17 +3201,15 @@
         <v>15</v>
       </c>
       <c r="B19">
-        <f>(MIN(C19,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C19-FARMER_HOURS)*TEMP_WORKER_RATE)+(A19*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C19-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A19*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>222195.97619685059</v>
       </c>
       <c r="C19">
-        <f>A19*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A19</f>
+        <f t="shared" si="1"/>
         <v>5639.2850287111351</v>
       </c>
       <c r="D19" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>31426.056999522843</v>
       </c>
     </row>
@@ -3249,17 +3218,15 @@
         <v>16</v>
       </c>
       <c r="B20">
-        <f>(MIN(C20,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C20-FARMER_HOURS)*TEMP_WORKER_RATE)+(A20*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C20-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A20*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>257893.94540430469</v>
       </c>
       <c r="C20">
-        <f>A20*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A20</f>
+        <f t="shared" si="1"/>
         <v>6616.761100354398</v>
       </c>
       <c r="D20" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>35697.969207454094</v>
       </c>
     </row>
@@ -3268,17 +3235,15 @@
         <v>17</v>
       </c>
       <c r="B21">
-        <f>(MIN(C21,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C21-FARMER_HOURS)*TEMP_WORKER_RATE)+(A21*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C21-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A21*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>298421.54869128112</v>
       </c>
       <c r="C21">
-        <f>A21*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A21</f>
+        <f t="shared" si="1"/>
         <v>7733.3395360392033</v>
       </c>
       <c r="D21" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>40527.603286976431</v>
       </c>
     </row>
@@ -3287,17 +3252,15 @@
         <v>18</v>
       </c>
       <c r="B22">
-        <f>(MIN(C22,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C22-FARMER_HOURS)*TEMP_WORKER_RATE)+(A22*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C22-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A22*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>344405.33318160975</v>
       </c>
       <c r="C22">
-        <f>A22*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A22</f>
+        <f t="shared" si="1"/>
         <v>9007.0660478574246</v>
       </c>
       <c r="D22" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>45983.784490328631</v>
       </c>
     </row>
@@ -3306,17 +3269,15 @@
         <v>19</v>
       </c>
       <c r="B23">
-        <f>(MIN(C23,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C23-FARMER_HOURS)*TEMP_WORKER_RATE)+(A23*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C23-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A23*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>396548.85908309149</v>
       </c>
       <c r="C23">
-        <f>A23*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A23</f>
+        <f t="shared" si="1"/>
         <v>10458.204466678902</v>
       </c>
       <c r="D23" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>52143.525901481742</v>
       </c>
     </row>
@@ -3325,17 +3286,15 @@
         <v>20</v>
       </c>
       <c r="B24">
-        <f>(MIN(C24,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C24-FARMER_HOURS)*TEMP_WORKER_RATE)+(A24*TOMATO_FERTILIZER_PER_BED)
-+(MAX(0,C24-FARMER_HOURS)*TEMP_WORKER_RATE)
-+(A24*TOMATO_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="0"/>
         <v>455641.83683305327</v>
       </c>
       <c r="C24">
-        <f>A24*TOMATO_HRS_PER_BED*WEEKS*(1+TOMATO_DIM_PCT)^A24</f>
+        <f t="shared" si="1"/>
         <v>12109.499908786096</v>
       </c>
       <c r="D24" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>59092.977749961778</v>
       </c>
     </row>
@@ -3345,7 +3304,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="19"/>
+      <c r="A27" s="11"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
@@ -3380,11 +3339,11 @@
         <v>1</v>
       </c>
       <c r="B30">
-        <f>(MIN(C30,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C30-FARMER_HOURS)*TEMP_WORKER_RATE)+(A30*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" ref="B30:B49" si="3">(MIN(C30,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C30-FARMER_HOURS)*TEMP_WORKER_RATE)+(A30*CARROT_FERTILIZER_PER_BED)</f>
         <v>1507.2129439999999</v>
       </c>
       <c r="C30">
-        <f>A30*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A30</f>
+        <f t="shared" ref="C30:C49" si="4">A30*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A30</f>
         <v>30.737699999999997</v>
       </c>
       <c r="D30" t="s">
@@ -3396,11 +3355,11 @@
         <v>2</v>
       </c>
       <c r="B31">
-        <f>(MIN(C31,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C31-FARMER_HOURS)*TEMP_WORKER_RATE)+(A31*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>3067.7865351999994</v>
       </c>
       <c r="C31">
-        <f>A31*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A31</f>
+        <f t="shared" si="4"/>
         <v>63.012284999999991</v>
       </c>
       <c r="D31" s="4">
@@ -3413,15 +3372,15 @@
         <v>3</v>
       </c>
       <c r="B32">
-        <f>(MIN(C32,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C32-FARMER_HOURS)*TEMP_WORKER_RATE)+(A32*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>4683.7217978699991</v>
       </c>
       <c r="C32">
-        <f>A32*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A32</f>
+        <f t="shared" si="4"/>
         <v>96.881388187499979</v>
       </c>
       <c r="D32" s="4">
-        <f t="shared" ref="D32:D49" si="1">B32-B31</f>
+        <f t="shared" ref="D32:D49" si="5">B32-B31</f>
         <v>1615.9352626699997</v>
       </c>
     </row>
@@ -3430,15 +3389,15 @@
         <v>4</v>
       </c>
       <c r="B33">
-        <f>(MIN(C33,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C33-FARMER_HOURS)*TEMP_WORKER_RATE)+(A33*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>6357.0864570889989</v>
       </c>
       <c r="C33">
-        <f>A33*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A33</f>
+        <f t="shared" si="4"/>
         <v>132.40456385624998</v>
       </c>
       <c r="D33" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>1673.3646592189998</v>
       </c>
     </row>
@@ -3447,15 +3406,15 @@
         <v>5</v>
       </c>
       <c r="B34">
-        <f>(MIN(C34,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C34-FARMER_HOURS)*TEMP_WORKER_RATE)+(A34*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>8090.0170231452794</v>
       </c>
       <c r="C34">
-        <f>A34*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A34</f>
+        <f t="shared" si="4"/>
         <v>169.64334744082026</v>
       </c>
       <c r="D34" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>1732.9305660562804</v>
       </c>
     </row>
@@ -3464,15 +3423,15 @@
         <v>6</v>
       </c>
       <c r="B35">
-        <f>(MIN(C35,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C35-FARMER_HOURS)*TEMP_WORKER_RATE)+(A35*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>9884.7209384686921</v>
       </c>
       <c r="C35">
-        <f>A35*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A35</f>
+        <f t="shared" si="4"/>
         <v>208.66131735220887</v>
       </c>
       <c r="D35" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>1794.7039153234127</v>
       </c>
     </row>
@@ -3481,15 +3440,15 @@
         <v>7</v>
       </c>
       <c r="B36">
-        <f>(MIN(C36,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C36-FARMER_HOURS)*TEMP_WORKER_RATE)+(A36*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>11743.478788918812</v>
       </c>
       <c r="C36">
-        <f>A36*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A36</f>
+        <f t="shared" si="4"/>
         <v>249.52415866701648</v>
       </c>
       <c r="D36" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>1858.7578504501198</v>
       </c>
     </row>
@@ -3498,15 +3457,15 @@
         <v>8</v>
       </c>
       <c r="B37">
-        <f>(MIN(C37,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C37-FARMER_HOURS)*TEMP_WORKER_RATE)+(A37*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>13668.646581304893</v>
       </c>
       <c r="C37">
-        <f>A37*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A37</f>
+        <f t="shared" si="4"/>
         <v>292.29972872421928</v>
       </c>
       <c r="D37" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>1925.1677923860807</v>
       </c>
     </row>
@@ -3515,15 +3474,15 @@
         <v>9</v>
       </c>
       <c r="B38">
-        <f>(MIN(C38,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C38-FARMER_HOURS)*TEMP_WORKER_RATE)+(A38*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>15662.658089067203</v>
       </c>
       <c r="C38">
-        <f>A38*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A38</f>
+        <f t="shared" si="4"/>
         <v>337.05812468511533</v>
       </c>
       <c r="D38" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>1994.0115077623104</v>
       </c>
     </row>
@@ -3532,15 +3491,15 @@
         <v>10</v>
       </c>
       <c r="B39">
-        <f>(MIN(C39,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C39-FARMER_HOURS)*TEMP_WORKER_RATE)+(A39*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>17728.027268104313</v>
       </c>
       <c r="C39">
-        <f>A39*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A39</f>
+        <f t="shared" si="4"/>
         <v>383.87175311360357</v>
       </c>
       <c r="D39" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>2065.3691790371104</v>
       </c>
     </row>
@@ -3549,15 +3508,15 @@
         <v>11</v>
       </c>
       <c r="B40">
-        <f>(MIN(C40,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C40-FARMER_HOURS)*TEMP_WORKER_RATE)+(A40*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>19867.350744787615</v>
       </c>
       <c r="C40">
-        <f>A40*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A40</f>
+        <f t="shared" si="4"/>
         <v>432.81540163558799</v>
       </c>
       <c r="D40" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>2139.3234766833011</v>
       </c>
     </row>
@@ -3566,15 +3525,15 @@
         <v>12</v>
       </c>
       <c r="B41">
-        <f>(MIN(C41,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C41-FARMER_HOURS)*TEMP_WORKER_RATE)+(A41*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>22083.310378262511</v>
       </c>
       <c r="C41">
-        <f>A41*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A41</f>
+        <f t="shared" si="4"/>
         <v>483.96631273797556</v>
       </c>
       <c r="D41" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>2215.9596334748967</v>
       </c>
     </row>
@@ -3583,15 +3542,15 @@
         <v>13</v>
       </c>
       <c r="B42">
-        <f>(MIN(C42,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C42-FARMER_HOURS)*TEMP_WORKER_RATE)+(A42*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>24378.675899195663</v>
       </c>
       <c r="C42">
-        <f>A42*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A42</f>
+        <f t="shared" si="4"/>
         <v>537.4042597694604</v>
       </c>
       <c r="D42" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>2295.3655209331519</v>
       </c>
     </row>
@@ -3600,15 +3559,15 @@
         <v>14</v>
       </c>
       <c r="B43">
-        <f>(MIN(C43,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C43-FARMER_HOURS)*TEMP_WORKER_RATE)+(A43*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>26756.30762718906</v>
       </c>
       <c r="C43">
-        <f>A43*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A43</f>
+        <f t="shared" si="4"/>
         <v>593.2116252070582</v>
       </c>
       <c r="D43" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>2377.6317279933974</v>
       </c>
     </row>
@@ -3617,15 +3576,15 @@
         <v>15</v>
       </c>
       <c r="B44">
-        <f>(MIN(C44,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C44-FARMER_HOURS)*TEMP_WORKER_RATE)+(A44*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>29219.15926914513</v>
       </c>
       <c r="C44">
-        <f>A44*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A44</f>
+        <f t="shared" si="4"/>
         <v>651.47348125418</v>
       </c>
       <c r="D44" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>2462.8516419560692</v>
       </c>
     </row>
@@ -3634,15 +3593,15 @@
         <v>16</v>
       </c>
       <c r="B45">
-        <f>(MIN(C45,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C45-FARMER_HOURS)*TEMP_WORKER_RATE)+(A45*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>31770.280800932007</v>
       </c>
       <c r="C45">
-        <f>A45*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A45</f>
+        <f t="shared" si="4"/>
         <v>712.27767283790342</v>
       </c>
       <c r="D45" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>2551.1215317868773</v>
       </c>
     </row>
@@ -3651,15 +3610,15 @@
         <v>17</v>
       </c>
       <c r="B46">
-        <f>(MIN(C46,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C46-FARMER_HOURS)*TEMP_WORKER_RATE)+(A46*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>33445.6107173825</v>
       </c>
       <c r="C46">
-        <f>A46*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A46</f>
+        <f t="shared" si="4"/>
         <v>775.71490307502916</v>
       </c>
       <c r="D46" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>1675.3299164504933</v>
       </c>
     </row>
@@ -3668,15 +3627,15 @@
         <v>18</v>
       </c>
       <c r="B47">
-        <f>(MIN(C47,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C47-FARMER_HOURS)*TEMP_WORKER_RATE)+(A47*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>35034.216337394537</v>
       </c>
       <c r="C47">
-        <f>A47*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A47</f>
+        <f t="shared" si="4"/>
         <v>841.87882127848752</v>
       </c>
       <c r="D47" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>1588.6056200120365</v>
       </c>
     </row>
@@ -3685,15 +3644,15 @@
         <v>19</v>
       </c>
       <c r="B48">
-        <f>(MIN(C48,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C48-FARMER_HOURS)*TEMP_WORKER_RATE)+(A48*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>36671.835731708816</v>
       </c>
       <c r="C48">
-        <f>A48*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A48</f>
+        <f t="shared" si="4"/>
         <v>910.86611357769698</v>
       </c>
       <c r="D48" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>1637.6193943142789</v>
       </c>
     </row>
@@ -3702,15 +3661,15 @@
         <v>20</v>
       </c>
       <c r="B49">
-        <f>(MIN(C49,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C49-FARMER_HOURS)*TEMP_WORKER_RATE)+(A49*CARROT_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="3"/>
         <v>38360.20171052793</v>
       </c>
       <c r="C49">
-        <f>A49*CARROT_HRS_PER_BED*WEEKS*(1+CARROT_DIM_PCT)^A49</f>
+        <f t="shared" si="4"/>
         <v>982.77659622856766</v>
       </c>
       <c r="D49" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>1688.3659788191144</v>
       </c>
     </row>
@@ -3719,11 +3678,11 @@
         <v>128</v>
       </c>
     </row>
-    <row r="52" spans="1:4" s="17" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A52" s="16"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="18" t="s">
+      <c r="A53" s="17" t="s">
         <v>137</v>
       </c>
       <c r="B53" s="5" t="s">
@@ -3737,7 +3696,7 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="18">
+      <c r="A54" s="17">
         <v>0</v>
       </c>
       <c r="B54" s="5">
@@ -3755,11 +3714,11 @@
         <v>1</v>
       </c>
       <c r="B55">
-        <f>(MIN(C55,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C55-FARMER_HOURS)*TEMP_WORKER_RATE)+(A55*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" ref="B55:B84" si="6">(MIN(C55,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C55-FARMER_HOURS)*TEMP_WORKER_RATE)+(A55*MESCLUN_FERTILIZER_PER_BED)</f>
         <v>2461.9299999999998</v>
       </c>
       <c r="C55" s="4">
-        <f>A55*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A55</f>
+        <f t="shared" ref="C55:C84" si="7">A55*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A55</f>
         <v>45.5625</v>
       </c>
       <c r="D55" t="s">
@@ -3771,11 +3730,11 @@
         <v>2</v>
       </c>
       <c r="B56">
-        <f>(MIN(C56,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C56-FARMER_HOURS)*TEMP_WORKER_RATE)+(A56*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>4963.4082499999995</v>
       </c>
       <c r="C56" s="4">
-        <f>A56*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A56</f>
+        <f t="shared" si="7"/>
         <v>92.264062499999994</v>
       </c>
       <c r="D56" s="4">
@@ -3788,15 +3747,15 @@
         <v>3</v>
       </c>
       <c r="B57">
-        <f>(MIN(C57,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C57-FARMER_HOURS)*TEMP_WORKER_RATE)+(A57*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>7505.1762796874991</v>
       </c>
       <c r="C57" s="4">
-        <f>A57*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A57</f>
+        <f t="shared" si="7"/>
         <v>140.12604492187498</v>
       </c>
       <c r="D57" s="4">
-        <f t="shared" ref="D57:D84" si="2">B57-B56</f>
+        <f t="shared" ref="D57:D84" si="8">B57-B56</f>
         <v>2541.7680296874996</v>
       </c>
     </row>
@@ -3805,15 +3764,15 @@
         <v>4</v>
       </c>
       <c r="B58">
-        <f>(MIN(C58,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C58-FARMER_HOURS)*TEMP_WORKER_RATE)+(A58*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>10087.987977578125</v>
       </c>
       <c r="C58" s="4">
-        <f>A58*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A58</f>
+        <f t="shared" si="7"/>
         <v>189.17016064453125</v>
       </c>
       <c r="D58" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2582.8116978906255</v>
       </c>
     </row>
@@ -3822,15 +3781,15 @@
         <v>5</v>
       </c>
       <c r="B59">
-        <f>(MIN(C59,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C59-FARMER_HOURS)*TEMP_WORKER_RATE)+(A59*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>12712.609784122313</v>
       </c>
       <c r="C59" s="4">
-        <f>A59*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A59</f>
+        <f t="shared" si="7"/>
         <v>239.41848456573481</v>
       </c>
       <c r="D59" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2624.6218065441881</v>
       </c>
     </row>
@@ -3839,15 +3798,15 @@
         <v>6</v>
       </c>
       <c r="B60">
-        <f>(MIN(C60,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C60-FARMER_HOURS)*TEMP_WORKER_RATE)+(A60*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>15379.820887708611</v>
       </c>
       <c r="C60" s="4">
-        <f>A60*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A60</f>
+        <f t="shared" si="7"/>
         <v>290.89345874736784</v>
       </c>
       <c r="D60" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2667.2111035862981</v>
       </c>
     </row>
@@ -3856,15 +3815,15 @@
         <v>7</v>
       </c>
       <c r="B61">
-        <f>(MIN(C61,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C61-FARMER_HOURS)*TEMP_WORKER_RATE)+(A61*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>18090.413423605794</v>
       </c>
       <c r="C61" s="4">
-        <f>A61*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A61</f>
+        <f t="shared" si="7"/>
         <v>343.61789814532818</v>
       </c>
       <c r="D61" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2710.5925358971836</v>
       </c>
     </row>
@@ -3873,15 +3832,15 @@
         <v>8</v>
       </c>
       <c r="B62">
-        <f>(MIN(C62,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C62-FARMER_HOURS)*TEMP_WORKER_RATE)+(A62*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>20845.192675886705</v>
       </c>
       <c r="C62" s="4">
-        <f>A62*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A62</f>
+        <f t="shared" si="7"/>
         <v>397.61499642530839</v>
       </c>
       <c r="D62" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2754.7792522809104</v>
       </c>
     </row>
@@ -3890,15 +3849,15 @@
         <v>9</v>
       </c>
       <c r="B63">
-        <f>(MIN(C63,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C63-FARMER_HOURS)*TEMP_WORKER_RATE)+(A63*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>23644.9772823772</v>
       </c>
       <c r="C63" s="4">
-        <f>A63*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A63</f>
+        <f t="shared" si="7"/>
         <v>452.90833186570285</v>
       </c>
       <c r="D63" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2799.7846064904952</v>
       </c>
     </row>
@@ -3907,15 +3866,15 @@
         <v>10</v>
       </c>
       <c r="B64">
-        <f>(MIN(C64,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C64-FARMER_HOURS)*TEMP_WORKER_RATE)+(A64*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>26490.599442674353</v>
       </c>
       <c r="C64" s="4">
-        <f>A64*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A64</f>
+        <f t="shared" si="7"/>
         <v>509.52187334891573</v>
       </c>
       <c r="D64" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2845.6221602971527</v>
       </c>
     </row>
@@ -3924,15 +3883,15 @@
         <v>11</v>
       </c>
       <c r="B65">
-        <f>(MIN(C65,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C65-FARMER_HOURS)*TEMP_WORKER_RATE)+(A65*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>29382.905129278555</v>
       </c>
       <c r="C65" s="4">
-        <f>A65*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A65</f>
+        <f t="shared" si="7"/>
         <v>567.47998644235474</v>
       </c>
       <c r="D65" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2892.3056866042025</v>
       </c>
     </row>
@@ -3941,15 +3900,15 @@
         <v>12</v>
       </c>
       <c r="B66">
-        <f>(MIN(C66,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C66-FARMER_HOURS)*TEMP_WORKER_RATE)+(A66*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>32322.754301884954</v>
       </c>
       <c r="C66" s="4">
-        <f>A66*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A66</f>
+        <f t="shared" si="7"/>
         <v>626.80743957041921</v>
       </c>
       <c r="D66" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2939.8491726063985</v>
       </c>
     </row>
@@ -3958,15 +3917,15 @@
         <v>13</v>
       </c>
       <c r="B67">
-        <f>(MIN(C67,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C67-FARMER_HOURS)*TEMP_WORKER_RATE)+(A67*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>35311.021124880055</v>
       </c>
       <c r="C67" s="4">
-        <f>A67*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A67</f>
+        <f t="shared" si="7"/>
         <v>687.52941027880343</v>
       </c>
       <c r="D67" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2988.2668229951014</v>
       </c>
     </row>
@@ -3975,15 +3934,15 @@
         <v>14</v>
       </c>
       <c r="B68">
-        <f>(MIN(C68,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C68-FARMER_HOURS)*TEMP_WORKER_RATE)+(A68*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>37833.497094045189</v>
       </c>
       <c r="C68" s="4">
-        <f>A68*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A68</f>
+        <f t="shared" si="7"/>
         <v>749.67149159246469</v>
       </c>
       <c r="D68" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2522.4759691651343</v>
       </c>
     </row>
@@ -3992,15 +3951,15 @@
         <v>15</v>
       </c>
       <c r="B69">
-        <f>(MIN(C69,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C69-FARMER_HOURS)*TEMP_WORKER_RATE)+(A69*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>39817.388365415085</v>
       </c>
       <c r="C69" s="4">
-        <f>A69*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A69</f>
+        <f t="shared" si="7"/>
         <v>813.25969846861108</v>
       </c>
       <c r="D69" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>1983.8912713698955</v>
       </c>
     </row>
@@ -4009,15 +3968,15 @@
         <v>16</v>
       </c>
       <c r="B70">
-        <f>(MIN(C70,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C70-FARMER_HOURS)*TEMP_WORKER_RATE)+(A70*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>41826.843434648297</v>
       </c>
       <c r="C70" s="4">
-        <f>A70*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A70</f>
+        <f t="shared" si="7"/>
         <v>878.32047434610013</v>
       </c>
       <c r="D70" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2009.4550692332123</v>
       </c>
     </row>
@@ -4026,15 +3985,15 @@
         <v>17</v>
       </c>
       <c r="B71">
-        <f>(MIN(C71,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C71-FARMER_HOURS)*TEMP_WORKER_RATE)+(A71*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>43862.328913680234</v>
       </c>
       <c r="C71" s="4">
-        <f>A71*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A71</f>
+        <f t="shared" si="7"/>
         <v>944.88069779264049</v>
       </c>
       <c r="D71" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2035.4854790319368</v>
       </c>
     </row>
@@ -4043,15 +4002,15 @@
         <v>18</v>
       </c>
       <c r="B72">
-        <f>(MIN(C72,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C72-FARMER_HOURS)*TEMP_WORKER_RATE)+(A72*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>45924.319085401308</v>
       </c>
       <c r="C72" s="4">
-        <f>A72*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A72</f>
+        <f t="shared" si="7"/>
         <v>1012.9676892512279</v>
       </c>
       <c r="D72" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2061.9901717210741</v>
       </c>
     </row>
@@ -4060,15 +4019,15 @@
         <v>19</v>
       </c>
       <c r="B73">
-        <f>(MIN(C73,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C73-FARMER_HOURS)*TEMP_WORKER_RATE)+(A73*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>48013.296022522649</v>
       </c>
       <c r="C73" s="4">
-        <f>A73*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A73</f>
+        <f t="shared" si="7"/>
         <v>1082.6092178872495</v>
       </c>
       <c r="D73" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2088.9769371213406</v>
       </c>
     </row>
@@ -4077,15 +4036,15 @@
         <v>20</v>
       </c>
       <c r="B74">
-        <f>(MIN(C74,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C74-FARMER_HOURS)*TEMP_WORKER_RATE)+(A74*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>50129.749708214935</v>
       </c>
       <c r="C74" s="4">
-        <f>A74*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A74</f>
+        <f t="shared" si="7"/>
         <v>1153.8335085377266</v>
       </c>
       <c r="D74" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2116.4536856922859</v>
       </c>
     </row>
@@ -4094,15 +4053,15 @@
         <v>21</v>
       </c>
       <c r="B75">
-        <f>(MIN(C75,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C75-FARMER_HOURS)*TEMP_WORKER_RATE)+(A75*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>52274.178158545998</v>
       </c>
       <c r="C75" s="4">
-        <f>A75*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A75</f>
+        <f t="shared" si="7"/>
         <v>1226.6692487641703</v>
       </c>
       <c r="D75" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2144.4284503310628</v>
       </c>
     </row>
@@ -4111,15 +4070,15 @@
         <v>22</v>
       </c>
       <c r="B76">
-        <f>(MIN(C76,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C76-FARMER_HOURS)*TEMP_WORKER_RATE)+(A76*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>54447.087546743431</v>
       </c>
       <c r="C76" s="4">
-        <f>A76*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A76</f>
+        <f t="shared" si="7"/>
         <v>1301.1455960105666</v>
       </c>
       <c r="D76" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2172.9093881974331</v>
       </c>
     </row>
@@ -4128,15 +4087,15 @@
         <v>23</v>
       </c>
       <c r="B77">
-        <f>(MIN(C77,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C77-FARMER_HOURS)*TEMP_WORKER_RATE)+(A77*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>56648.99232930853</v>
       </c>
       <c r="C77" s="4">
-        <f>A77*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A77</f>
+        <f t="shared" si="7"/>
         <v>1377.292184868003</v>
       </c>
       <c r="D77" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2201.9047825650996</v>
       </c>
     </row>
@@ -4145,15 +4104,15 @@
         <v>24</v>
       </c>
       <c r="B78">
-        <f>(MIN(C78,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C78-FARMER_HOURS)*TEMP_WORKER_RATE)+(A78*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>58880.415374008575</v>
       </c>
       <c r="C78" s="4">
-        <f>A78*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A78</f>
+        <f t="shared" si="7"/>
         <v>1455.1391344474989</v>
       </c>
       <c r="D78" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2231.4230447000446</v>
       </c>
     </row>
@@ -4162,15 +4121,15 @@
         <v>25</v>
       </c>
       <c r="B79">
-        <f>(MIN(C79,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C79-FARMER_HOURS)*TEMP_WORKER_RATE)+(A79*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>61141.888089774671</v>
       </c>
       <c r="C79" s="4">
-        <f>A79*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A79</f>
+        <f t="shared" si="7"/>
         <v>1534.7170558625965</v>
       </c>
       <c r="D79" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2261.4727157660964</v>
       </c>
     </row>
@@ -4179,15 +4138,15 @@
         <v>26</v>
       </c>
       <c r="B80">
-        <f>(MIN(C80,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C80-FARMER_HOURS)*TEMP_WORKER_RATE)+(A80*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>63433.950558532735</v>
       </c>
       <c r="C80" s="4">
-        <f>A80*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A80</f>
+        <f t="shared" si="7"/>
         <v>1616.0570598233144</v>
       </c>
       <c r="D80" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2292.0624687580639</v>
       </c>
     </row>
@@ -4196,15 +4155,15 @@
         <v>27</v>
       </c>
       <c r="B81">
-        <f>(MIN(C81,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C81-FARMER_HOURS)*TEMP_WORKER_RATE)+(A81*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>65757.151668995706</v>
       </c>
       <c r="C81" s="4">
-        <f>A81*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A81</f>
+        <f t="shared" si="7"/>
         <v>1699.1907643430709</v>
       </c>
       <c r="D81" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2323.201110462971</v>
       </c>
     </row>
@@ -4213,15 +4172,15 @@
         <v>28</v>
       </c>
       <c r="B82">
-        <f>(MIN(C82,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C82-FARMER_HOURS)*TEMP_WORKER_RATE)+(A82*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>68112.049252445489</v>
       </c>
       <c r="C82" s="4">
-        <f>A82*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A82</f>
+        <f t="shared" si="7"/>
         <v>1784.1503025602246</v>
       </c>
       <c r="D82" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2354.8975834497833</v>
       </c>
     </row>
@@ -4230,15 +4189,15 @@
         <v>29</v>
       </c>
       <c r="B83">
-        <f>(MIN(C83,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C83-FARMER_HOURS)*TEMP_WORKER_RATE)+(A83*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>70499.210220533249</v>
       </c>
       <c r="C83" s="4">
-        <f>A83*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A83</f>
+        <f t="shared" si="7"/>
         <v>1870.9683306758782</v>
       </c>
       <c r="D83" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2387.1609680877591</v>
       </c>
     </row>
@@ -4247,15 +4206,15 @@
         <v>30</v>
       </c>
       <c r="B84">
-        <f>(MIN(C84,FARMER_HOURS)*FARMER_RATE)+(MAX(0,C84-FARMER_HOURS)*TEMP_WORKER_RATE)+(A84*MESCLUN_FERTILIZER_PER_BED)</f>
+        <f t="shared" si="6"/>
         <v>72919.210705127509</v>
       </c>
       <c r="C84" s="4">
-        <f>A84*MESCLUN_HRS_PER_BED*WEEKS*(1+MESCLUN_DIM_PCT)^A84</f>
+        <f t="shared" si="7"/>
         <v>1959.6780360096488</v>
       </c>
       <c r="D84" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>2420.0004845942603</v>
       </c>
     </row>

</xml_diff>